<commit_message>
Hydraulics: Mach/ρv² outputs and manual stream composition with mixing
- Pressure_Profile and FIV_EI_T2.2: add Mach (vapor), ρv² vapor and ρv² liquid
  per station (phase superficial velocities; vapor sound speed from Cp/Cv, Z, T, MW).
- New Stream_Composition input sheet: vapor/liquid mass or mole composition per
  Line/Seq for runs that do not reference an HMB stream. Component MW/Tc/Pc/ω come
  from the HMB COMP_CONSTANTS sheet. First composition starts the flow; later
  ones (other Seq or extra columns) are mixed in and re-flashed.
- Template, Notes and README updated; hydraulics.py brought up to the latest
  uploaded version (26-36 in sizes, Tee Split/Join Branch Flow 3-6, overrides).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016tUfEsTN4BKrSujrNZ7fBp
</commit_message>
<xml_diff>
--- a/Hydraulics/pipeline_input_noiso.xlsx
+++ b/Hydraulics/pipeline_input_noiso.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Pipeline_Input" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="_FittingList" sheetId="2" state="hidden" r:id="rId2"/>
-    <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="UNITS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline_Input" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_FittingList" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stream_Composition" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UNITS" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pipeline_Input'!$A$2:$AK$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pipeline_Input'!$A$2:$AM$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -50,13 +51,13 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001F4973"/>
+      <color rgb="00404040"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00404040"/>
+      <b val="1"/>
+      <color rgb="001F4973"/>
       <sz val="9"/>
     </font>
     <font>
@@ -82,7 +83,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -102,6 +103,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00375623"/>
       </patternFill>
     </fill>
     <fill>
@@ -136,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -150,12 +156,30 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -167,7 +191,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -541,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK20"/>
+  <dimension ref="A1:AM20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -553,34 +577,36 @@
     <col width="6" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="9" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="8" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="10" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
-    <col width="32" customWidth="1" min="23" max="23"/>
-    <col width="9" customWidth="1" min="24" max="24"/>
-    <col width="11" customWidth="1" min="25" max="25"/>
-    <col width="11" customWidth="1" min="26" max="26"/>
-    <col width="13" customWidth="1" min="27" max="27"/>
-    <col width="10" customWidth="1" min="28" max="28"/>
-    <col width="9" customWidth="1" min="29" max="29"/>
-    <col width="12" customWidth="1" min="30" max="30"/>
-    <col width="10" customWidth="1" min="31" max="31"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="32" customWidth="1" min="25" max="25"/>
+    <col width="9" customWidth="1" min="26" max="26"/>
+    <col width="11" customWidth="1" min="27" max="27"/>
+    <col width="11" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="29" max="29"/>
+    <col width="10" customWidth="1" min="30" max="30"/>
+    <col width="9" customWidth="1" min="31" max="31"/>
     <col width="12" customWidth="1" min="32" max="32"/>
-    <col width="12" customWidth="1" min="33" max="33"/>
+    <col width="10" customWidth="1" min="33" max="33"/>
     <col width="12" customWidth="1" min="34" max="34"/>
-    <col width="14" customWidth="1" min="35" max="35"/>
-    <col width="16" customWidth="1" min="36" max="36"/>
-    <col width="30" customWidth="1" min="37" max="37"/>
+    <col width="12" customWidth="1" min="35" max="35"/>
+    <col width="12" customWidth="1" min="36" max="36"/>
+    <col width="14" customWidth="1" min="37" max="37"/>
+    <col width="16" customWidth="1" min="38" max="38"/>
+    <col width="30" customWidth="1" min="39" max="39"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -633,145 +659,155 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
+          <t>Upstream Line No</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Upstream Seq</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
           <t>Flow Fraction from Main</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Mass Vapor Fraction Carry Over</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Mass Liquid Fraction Carry Over</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Temp (°F)</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>Vapor Mass Flow (lb/hr)</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Vap MW</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>Vap Visc (cP)</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>Vap Z</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>Vap Cp/Cv</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>Vap Density (lb/ft3)</t>
         </is>
       </c>
-      <c r="S2" s="2" t="inlineStr">
+      <c r="U2" s="2" t="inlineStr">
         <is>
           <t>Liq Mass Flow (lb/hr)</t>
         </is>
       </c>
-      <c r="T2" s="2" t="inlineStr">
+      <c r="V2" s="2" t="inlineStr">
         <is>
           <t>Liq Density (lb/ft3)</t>
         </is>
       </c>
-      <c r="U2" s="2" t="inlineStr">
+      <c r="W2" s="2" t="inlineStr">
         <is>
           <t>Liq Visc (cP)</t>
         </is>
       </c>
-      <c r="V2" s="2" t="inlineStr">
+      <c r="X2" s="2" t="inlineStr">
         <is>
           <t>Comp ID</t>
         </is>
       </c>
-      <c r="W2" s="2" t="inlineStr">
+      <c r="Y2" s="2" t="inlineStr">
         <is>
           <t>Fitting Name</t>
         </is>
       </c>
-      <c r="X2" s="2" t="inlineStr">
+      <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>Bore (in)</t>
         </is>
       </c>
-      <c r="Y2" s="2" t="inlineStr">
+      <c r="AA2" s="2" t="inlineStr">
         <is>
           <t>Piping Spec</t>
         </is>
       </c>
-      <c r="Z2" s="2" t="inlineStr">
+      <c r="AB2" s="2" t="inlineStr">
         <is>
           <t>Length (ft)</t>
         </is>
       </c>
-      <c r="AA2" s="2" t="inlineStr">
+      <c r="AC2" s="2" t="inlineStr">
         <is>
           <t>Elev Change (ft)</t>
         </is>
       </c>
-      <c r="AB2" s="2" t="inlineStr">
+      <c r="AD2" s="2" t="inlineStr">
         <is>
           <t>Direction</t>
         </is>
       </c>
-      <c r="AC2" s="2" t="inlineStr">
+      <c r="AE2" s="2" t="inlineStr">
         <is>
           <t>Fixed K</t>
         </is>
       </c>
-      <c r="AD2" s="2" t="inlineStr">
+      <c r="AF2" s="2" t="inlineStr">
         <is>
           <t>Fixed dP (psi)</t>
         </is>
       </c>
-      <c r="AE2" s="2" t="inlineStr">
+      <c r="AG2" s="2" t="inlineStr">
         <is>
           <t>Instr Type</t>
         </is>
       </c>
-      <c r="AF2" s="2" t="inlineStr">
+      <c r="AH2" s="2" t="inlineStr">
         <is>
           <t>Instr Tag</t>
         </is>
       </c>
-      <c r="AG2" s="2" t="inlineStr">
+      <c r="AI2" s="2" t="inlineStr">
         <is>
           <t>Instr dP (psi)</t>
         </is>
       </c>
-      <c r="AH2" s="2" t="inlineStr">
+      <c r="AJ2" s="2" t="inlineStr">
         <is>
           <t>Set P (psia)</t>
         </is>
       </c>
-      <c r="AI2" s="2" t="inlineStr">
+      <c r="AK2" s="2" t="inlineStr">
         <is>
           <t>Control Valve Type</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr">
+      <c r="AL2" s="2" t="inlineStr">
         <is>
           <t>Exch Max Allow dP (psi)</t>
         </is>
       </c>
-      <c r="AK2" s="2" t="inlineStr">
+      <c r="AM2" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -809,8 +845,8 @@
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
       <c r="K3" s="3" t="n"/>
-      <c r="L3" s="4" t="n"/>
-      <c r="M3" s="4" t="n"/>
+      <c r="L3" s="3" t="n"/>
+      <c r="M3" s="3" t="n"/>
       <c r="N3" s="4" t="n"/>
       <c r="O3" s="4" t="n"/>
       <c r="P3" s="4" t="n"/>
@@ -819,32 +855,32 @@
       <c r="S3" s="4" t="n"/>
       <c r="T3" s="4" t="n"/>
       <c r="U3" s="4" t="n"/>
-      <c r="V3" s="3" t="inlineStr">
+      <c r="V3" s="4" t="n"/>
+      <c r="W3" s="4" t="n"/>
+      <c r="X3" s="3" t="inlineStr">
         <is>
           <t>ENT-01</t>
         </is>
       </c>
-      <c r="W3" s="3" t="inlineStr">
+      <c r="Y3" s="3" t="inlineStr">
         <is>
           <t>Pipeline Entrance - Sharp Edge</t>
         </is>
       </c>
-      <c r="X3" s="3" t="n">
+      <c r="Z3" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="Y3" s="3" t="inlineStr">
+      <c r="AA3" s="3" t="inlineStr">
         <is>
           <t>G1A-5</t>
         </is>
       </c>
-      <c r="Z3" s="3" t="n">
+      <c r="AB3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AA3" s="3" t="n">
+      <c r="AC3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AB3" s="3" t="n"/>
-      <c r="AC3" s="3" t="n"/>
       <c r="AD3" s="3" t="n"/>
       <c r="AE3" s="3" t="n"/>
       <c r="AF3" s="3" t="n"/>
@@ -852,7 +888,9 @@
       <c r="AH3" s="3" t="n"/>
       <c r="AI3" s="3" t="n"/>
       <c r="AJ3" s="3" t="n"/>
-      <c r="AK3" s="3" t="inlineStr">
+      <c r="AK3" s="3" t="n"/>
+      <c r="AL3" s="3" t="n"/>
+      <c r="AM3" s="3" t="inlineStr">
         <is>
           <t>Entrance</t>
         </is>
@@ -884,8 +922,8 @@
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
       <c r="K4" s="3" t="n"/>
-      <c r="L4" s="4" t="n"/>
-      <c r="M4" s="4" t="n"/>
+      <c r="L4" s="3" t="n"/>
+      <c r="M4" s="3" t="n"/>
       <c r="N4" s="4" t="n"/>
       <c r="O4" s="4" t="n"/>
       <c r="P4" s="4" t="n"/>
@@ -894,44 +932,46 @@
       <c r="S4" s="4" t="n"/>
       <c r="T4" s="4" t="n"/>
       <c r="U4" s="4" t="n"/>
-      <c r="V4" s="3" t="inlineStr">
+      <c r="V4" s="4" t="n"/>
+      <c r="W4" s="4" t="n"/>
+      <c r="X4" s="3" t="inlineStr">
         <is>
           <t>P-001</t>
         </is>
       </c>
-      <c r="W4" s="3" t="inlineStr">
+      <c r="Y4" s="3" t="inlineStr">
         <is>
           <t>Straight Pipeline</t>
         </is>
       </c>
-      <c r="X4" s="3" t="n">
+      <c r="Z4" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="Y4" s="3" t="inlineStr">
+      <c r="AA4" s="3" t="inlineStr">
         <is>
           <t>G1A-5</t>
         </is>
       </c>
-      <c r="Z4" s="3" t="n">
+      <c r="AB4" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="AA4" s="3" t="n">
+      <c r="AC4" s="3" t="n">
         <v>-2</v>
       </c>
-      <c r="AB4" s="3" t="inlineStr">
+      <c r="AD4" s="3" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="AC4" s="3" t="n"/>
-      <c r="AD4" s="3" t="n"/>
       <c r="AE4" s="3" t="n"/>
       <c r="AF4" s="3" t="n"/>
       <c r="AG4" s="3" t="n"/>
       <c r="AH4" s="3" t="n"/>
       <c r="AI4" s="3" t="n"/>
       <c r="AJ4" s="3" t="n"/>
-      <c r="AK4" s="3" t="inlineStr">
+      <c r="AK4" s="3" t="n"/>
+      <c r="AL4" s="3" t="n"/>
+      <c r="AM4" s="3" t="inlineStr">
         <is>
           <t>Drop leg</t>
         </is>
@@ -963,8 +1003,8 @@
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
       <c r="K5" s="3" t="n"/>
-      <c r="L5" s="4" t="n"/>
-      <c r="M5" s="4" t="n"/>
+      <c r="L5" s="3" t="n"/>
+      <c r="M5" s="3" t="n"/>
       <c r="N5" s="4" t="n"/>
       <c r="O5" s="4" t="n"/>
       <c r="P5" s="4" t="n"/>
@@ -973,32 +1013,32 @@
       <c r="S5" s="4" t="n"/>
       <c r="T5" s="4" t="n"/>
       <c r="U5" s="4" t="n"/>
-      <c r="V5" s="3" t="inlineStr">
+      <c r="V5" s="4" t="n"/>
+      <c r="W5" s="4" t="n"/>
+      <c r="X5" s="3" t="inlineStr">
         <is>
           <t>EL-001</t>
         </is>
       </c>
-      <c r="W5" s="3" t="inlineStr">
+      <c r="Y5" s="3" t="inlineStr">
         <is>
           <t>Elbow 90 Long</t>
         </is>
       </c>
-      <c r="X5" s="3" t="n">
+      <c r="Z5" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="Y5" s="3" t="inlineStr">
+      <c r="AA5" s="3" t="inlineStr">
         <is>
           <t>G1A-5</t>
         </is>
       </c>
-      <c r="Z5" s="3" t="n">
+      <c r="AB5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AA5" s="3" t="n">
+      <c r="AC5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AB5" s="3" t="n"/>
-      <c r="AC5" s="3" t="n"/>
       <c r="AD5" s="3" t="n"/>
       <c r="AE5" s="3" t="n"/>
       <c r="AF5" s="3" t="n"/>
@@ -1007,6 +1047,8 @@
       <c r="AI5" s="3" t="n"/>
       <c r="AJ5" s="3" t="n"/>
       <c r="AK5" s="3" t="n"/>
+      <c r="AL5" s="3" t="n"/>
+      <c r="AM5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1031,13 +1073,13 @@
         <v>4</v>
       </c>
       <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n">
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
+      <c r="K6" s="3" t="n">
         <v>-0.4</v>
       </c>
-      <c r="J6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="4" t="n"/>
-      <c r="M6" s="4" t="n"/>
+      <c r="L6" s="3" t="n"/>
+      <c r="M6" s="3" t="n"/>
       <c r="N6" s="4" t="n"/>
       <c r="O6" s="4" t="n"/>
       <c r="P6" s="4" t="n"/>
@@ -1046,32 +1088,32 @@
       <c r="S6" s="4" t="n"/>
       <c r="T6" s="4" t="n"/>
       <c r="U6" s="4" t="n"/>
-      <c r="V6" s="3" t="inlineStr">
+      <c r="V6" s="4" t="n"/>
+      <c r="W6" s="4" t="n"/>
+      <c r="X6" s="3" t="inlineStr">
         <is>
           <t>TEE-01</t>
         </is>
       </c>
-      <c r="W6" s="3" t="inlineStr">
+      <c r="Y6" s="3" t="inlineStr">
         <is>
           <t>Tee Split Line Flow</t>
         </is>
       </c>
-      <c r="X6" s="3" t="n">
+      <c r="Z6" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="Y6" s="3" t="inlineStr">
+      <c r="AA6" s="3" t="inlineStr">
         <is>
           <t>G1A-5</t>
         </is>
       </c>
-      <c r="Z6" s="3" t="n">
+      <c r="AB6" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AA6" s="3" t="n">
+      <c r="AC6" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AB6" s="3" t="n"/>
-      <c r="AC6" s="3" t="n"/>
       <c r="AD6" s="3" t="n"/>
       <c r="AE6" s="3" t="n"/>
       <c r="AF6" s="3" t="n"/>
@@ -1079,7 +1121,9 @@
       <c r="AH6" s="3" t="n"/>
       <c r="AI6" s="3" t="n"/>
       <c r="AJ6" s="3" t="n"/>
-      <c r="AK6" s="3" t="inlineStr">
+      <c r="AK6" s="3" t="n"/>
+      <c r="AL6" s="3" t="n"/>
+      <c r="AM6" s="3" t="inlineStr">
         <is>
           <t>40% splits to branch</t>
         </is>
@@ -1111,8 +1155,8 @@
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
       <c r="K7" s="3" t="n"/>
-      <c r="L7" s="4" t="n"/>
-      <c r="M7" s="4" t="n"/>
+      <c r="L7" s="3" t="n"/>
+      <c r="M7" s="3" t="n"/>
       <c r="N7" s="4" t="n"/>
       <c r="O7" s="4" t="n"/>
       <c r="P7" s="4" t="n"/>
@@ -1121,42 +1165,44 @@
       <c r="S7" s="4" t="n"/>
       <c r="T7" s="4" t="n"/>
       <c r="U7" s="4" t="n"/>
-      <c r="V7" s="3" t="inlineStr">
+      <c r="V7" s="4" t="n"/>
+      <c r="W7" s="4" t="n"/>
+      <c r="X7" s="3" t="inlineStr">
         <is>
           <t>PSV-01</t>
         </is>
       </c>
-      <c r="W7" s="3" t="inlineStr">
+      <c r="Y7" s="3" t="inlineStr">
         <is>
           <t>Fix Pressure</t>
         </is>
       </c>
-      <c r="X7" s="3" t="n">
+      <c r="Z7" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="Y7" s="3" t="inlineStr">
+      <c r="AA7" s="3" t="inlineStr">
         <is>
           <t>G1A-5</t>
         </is>
       </c>
-      <c r="Z7" s="3" t="n">
+      <c r="AB7" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AA7" s="3" t="n">
+      <c r="AC7" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AB7" s="3" t="n"/>
-      <c r="AC7" s="3" t="n"/>
-      <c r="AD7" s="3" t="n">
+      <c r="AD7" s="3" t="n"/>
+      <c r="AE7" s="3" t="n"/>
+      <c r="AF7" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="AE7" s="3" t="n"/>
-      <c r="AF7" s="3" t="n"/>
       <c r="AG7" s="3" t="n"/>
       <c r="AH7" s="3" t="n"/>
       <c r="AI7" s="3" t="n"/>
       <c r="AJ7" s="3" t="n"/>
-      <c r="AK7" s="3" t="inlineStr">
+      <c r="AK7" s="3" t="n"/>
+      <c r="AL7" s="3" t="n"/>
+      <c r="AM7" s="3" t="inlineStr">
         <is>
           <t>PSV seat loss</t>
         </is>
@@ -1188,8 +1234,8 @@
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
       <c r="K8" s="3" t="n"/>
-      <c r="L8" s="4" t="n"/>
-      <c r="M8" s="4" t="n"/>
+      <c r="L8" s="3" t="n"/>
+      <c r="M8" s="3" t="n"/>
       <c r="N8" s="4" t="n"/>
       <c r="O8" s="4" t="n"/>
       <c r="P8" s="4" t="n"/>
@@ -1198,32 +1244,32 @@
       <c r="S8" s="4" t="n"/>
       <c r="T8" s="4" t="n"/>
       <c r="U8" s="4" t="n"/>
-      <c r="V8" s="3" t="inlineStr">
+      <c r="V8" s="4" t="n"/>
+      <c r="W8" s="4" t="n"/>
+      <c r="X8" s="3" t="inlineStr">
         <is>
           <t>P-002</t>
         </is>
       </c>
-      <c r="W8" s="3" t="inlineStr">
+      <c r="Y8" s="3" t="inlineStr">
         <is>
           <t>Straight Pipeline</t>
         </is>
       </c>
-      <c r="X8" s="3" t="n">
+      <c r="Z8" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="Y8" s="3" t="inlineStr">
+      <c r="AA8" s="3" t="inlineStr">
         <is>
           <t>G1A-5</t>
         </is>
       </c>
-      <c r="Z8" s="3" t="n">
+      <c r="AB8" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="AA8" s="3" t="n">
+      <c r="AC8" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AB8" s="3" t="n"/>
-      <c r="AC8" s="3" t="n"/>
       <c r="AD8" s="3" t="n"/>
       <c r="AE8" s="3" t="n"/>
       <c r="AF8" s="3" t="n"/>
@@ -1231,7 +1277,9 @@
       <c r="AH8" s="3" t="n"/>
       <c r="AI8" s="3" t="n"/>
       <c r="AJ8" s="3" t="n"/>
-      <c r="AK8" s="3" t="inlineStr">
+      <c r="AK8" s="3" t="n"/>
+      <c r="AL8" s="3" t="n"/>
+      <c r="AM8" s="3" t="inlineStr">
         <is>
           <t>Header run</t>
         </is>
@@ -1263,8 +1311,8 @@
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
       <c r="K9" s="3" t="n"/>
-      <c r="L9" s="4" t="n"/>
-      <c r="M9" s="4" t="n"/>
+      <c r="L9" s="3" t="n"/>
+      <c r="M9" s="3" t="n"/>
       <c r="N9" s="4" t="n"/>
       <c r="O9" s="4" t="n"/>
       <c r="P9" s="4" t="n"/>
@@ -1273,32 +1321,32 @@
       <c r="S9" s="4" t="n"/>
       <c r="T9" s="4" t="n"/>
       <c r="U9" s="4" t="n"/>
-      <c r="V9" s="3" t="inlineStr">
+      <c r="V9" s="4" t="n"/>
+      <c r="W9" s="4" t="n"/>
+      <c r="X9" s="3" t="inlineStr">
         <is>
           <t>EL-002</t>
         </is>
       </c>
-      <c r="W9" s="3" t="inlineStr">
+      <c r="Y9" s="3" t="inlineStr">
         <is>
           <t>Elbow 90 Long</t>
         </is>
       </c>
-      <c r="X9" s="3" t="n">
+      <c r="Z9" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="Y9" s="3" t="inlineStr">
+      <c r="AA9" s="3" t="inlineStr">
         <is>
           <t>G1A-5</t>
         </is>
       </c>
-      <c r="Z9" s="3" t="n">
+      <c r="AB9" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AA9" s="3" t="n">
+      <c r="AC9" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AB9" s="3" t="n"/>
-      <c r="AC9" s="3" t="n"/>
       <c r="AD9" s="3" t="n"/>
       <c r="AE9" s="3" t="n"/>
       <c r="AF9" s="3" t="n"/>
@@ -1307,6 +1355,8 @@
       <c r="AI9" s="3" t="n"/>
       <c r="AJ9" s="3" t="n"/>
       <c r="AK9" s="3" t="n"/>
+      <c r="AL9" s="3" t="n"/>
+      <c r="AM9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1334,8 +1384,8 @@
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
       <c r="K10" s="3" t="n"/>
-      <c r="L10" s="4" t="n"/>
-      <c r="M10" s="4" t="n"/>
+      <c r="L10" s="3" t="n"/>
+      <c r="M10" s="3" t="n"/>
       <c r="N10" s="4" t="n"/>
       <c r="O10" s="4" t="n"/>
       <c r="P10" s="4" t="n"/>
@@ -1344,42 +1394,44 @@
       <c r="S10" s="4" t="n"/>
       <c r="T10" s="4" t="n"/>
       <c r="U10" s="4" t="n"/>
-      <c r="V10" s="3" t="inlineStr">
+      <c r="V10" s="4" t="n"/>
+      <c r="W10" s="4" t="n"/>
+      <c r="X10" s="3" t="inlineStr">
         <is>
           <t>VLV-01</t>
         </is>
       </c>
-      <c r="W10" s="3" t="inlineStr">
+      <c r="Y10" s="3" t="inlineStr">
         <is>
           <t>Fix K</t>
         </is>
       </c>
-      <c r="X10" s="3" t="n">
+      <c r="Z10" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="Y10" s="3" t="inlineStr">
+      <c r="AA10" s="3" t="inlineStr">
         <is>
           <t>G1A-5</t>
         </is>
       </c>
-      <c r="Z10" s="3" t="n">
+      <c r="AB10" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AA10" s="3" t="n">
+      <c r="AC10" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AB10" s="3" t="n"/>
-      <c r="AC10" s="3" t="n">
+      <c r="AD10" s="3" t="n"/>
+      <c r="AE10" s="3" t="n">
         <v>7.2</v>
       </c>
-      <c r="AD10" s="3" t="n"/>
-      <c r="AE10" s="3" t="n"/>
       <c r="AF10" s="3" t="n"/>
       <c r="AG10" s="3" t="n"/>
       <c r="AH10" s="3" t="n"/>
       <c r="AI10" s="3" t="n"/>
       <c r="AJ10" s="3" t="n"/>
-      <c r="AK10" s="3" t="inlineStr">
+      <c r="AK10" s="3" t="n"/>
+      <c r="AL10" s="3" t="n"/>
+      <c r="AM10" s="3" t="inlineStr">
         <is>
           <t>CV K=7.2</t>
         </is>
@@ -1413,56 +1465,56 @@
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
       <c r="K11" s="3" t="n"/>
-      <c r="L11" s="4" t="n">
+      <c r="L11" s="3" t="n"/>
+      <c r="M11" s="3" t="n"/>
+      <c r="N11" s="4" t="n">
         <v>250</v>
       </c>
-      <c r="M11" s="4" t="n">
+      <c r="O11" s="4" t="n">
         <v>12000</v>
       </c>
-      <c r="N11" s="4" t="n">
+      <c r="P11" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="O11" s="4" t="n">
+      <c r="Q11" s="4" t="n">
         <v>0.012</v>
       </c>
-      <c r="P11" s="4" t="n">
+      <c r="R11" s="4" t="n">
         <v>0.95</v>
       </c>
-      <c r="Q11" s="4" t="n">
+      <c r="S11" s="4" t="n">
         <v>1.28</v>
       </c>
-      <c r="R11" s="4" t="n">
+      <c r="T11" s="4" t="n">
         <v>0.45</v>
       </c>
-      <c r="S11" s="4" t="n"/>
-      <c r="T11" s="4" t="n"/>
       <c r="U11" s="4" t="n"/>
-      <c r="V11" s="3" t="inlineStr">
+      <c r="V11" s="4" t="n"/>
+      <c r="W11" s="4" t="n"/>
+      <c r="X11" s="3" t="inlineStr">
         <is>
           <t>P-003</t>
         </is>
       </c>
-      <c r="W11" s="3" t="inlineStr">
+      <c r="Y11" s="3" t="inlineStr">
         <is>
           <t>Straight Pipeline</t>
         </is>
       </c>
-      <c r="X11" s="3" t="n">
+      <c r="Z11" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="Y11" s="3" t="inlineStr">
+      <c r="AA11" s="3" t="inlineStr">
         <is>
           <t>G1A-5</t>
         </is>
       </c>
-      <c r="Z11" s="3" t="n">
+      <c r="AB11" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="AA11" s="3" t="n">
+      <c r="AC11" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AB11" s="3" t="n"/>
-      <c r="AC11" s="3" t="n"/>
       <c r="AD11" s="3" t="n"/>
       <c r="AE11" s="3" t="n"/>
       <c r="AF11" s="3" t="n"/>
@@ -1470,7 +1522,9 @@
       <c r="AH11" s="3" t="n"/>
       <c r="AI11" s="3" t="n"/>
       <c r="AJ11" s="3" t="n"/>
-      <c r="AK11" s="3" t="inlineStr">
+      <c r="AK11" s="3" t="n"/>
+      <c r="AL11" s="3" t="n"/>
+      <c r="AM11" s="3" t="inlineStr">
         <is>
           <t>Manual props (no stream)</t>
         </is>
@@ -1502,8 +1556,8 @@
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
       <c r="K12" s="3" t="n"/>
-      <c r="L12" s="4" t="n"/>
-      <c r="M12" s="4" t="n"/>
+      <c r="L12" s="3" t="n"/>
+      <c r="M12" s="3" t="n"/>
       <c r="N12" s="4" t="n"/>
       <c r="O12" s="4" t="n"/>
       <c r="P12" s="4" t="n"/>
@@ -1512,32 +1566,32 @@
       <c r="S12" s="4" t="n"/>
       <c r="T12" s="4" t="n"/>
       <c r="U12" s="4" t="n"/>
-      <c r="V12" s="3" t="inlineStr">
+      <c r="V12" s="4" t="n"/>
+      <c r="W12" s="4" t="n"/>
+      <c r="X12" s="3" t="inlineStr">
         <is>
           <t>EL-003</t>
         </is>
       </c>
-      <c r="W12" s="3" t="inlineStr">
+      <c r="Y12" s="3" t="inlineStr">
         <is>
           <t>Elbow 90 Long</t>
         </is>
       </c>
-      <c r="X12" s="3" t="n">
+      <c r="Z12" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="Y12" s="3" t="inlineStr">
+      <c r="AA12" s="3" t="inlineStr">
         <is>
           <t>G1A-5</t>
         </is>
       </c>
-      <c r="Z12" s="3" t="n">
+      <c r="AB12" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AA12" s="3" t="n">
+      <c r="AC12" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AB12" s="3" t="n"/>
-      <c r="AC12" s="3" t="n"/>
       <c r="AD12" s="3" t="n"/>
       <c r="AE12" s="3" t="n"/>
       <c r="AF12" s="3" t="n"/>
@@ -1546,6 +1600,8 @@
       <c r="AI12" s="3" t="n"/>
       <c r="AJ12" s="3" t="n"/>
       <c r="AK12" s="3" t="n"/>
+      <c r="AL12" s="3" t="n"/>
+      <c r="AM12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1577,8 +1633,8 @@
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n"/>
       <c r="K13" s="3" t="n"/>
-      <c r="L13" s="4" t="n"/>
-      <c r="M13" s="4" t="n"/>
+      <c r="L13" s="3" t="n"/>
+      <c r="M13" s="3" t="n"/>
       <c r="N13" s="4" t="n"/>
       <c r="O13" s="4" t="n"/>
       <c r="P13" s="4" t="n"/>
@@ -1587,42 +1643,44 @@
       <c r="S13" s="4" t="n"/>
       <c r="T13" s="4" t="n"/>
       <c r="U13" s="4" t="n"/>
-      <c r="V13" s="3" t="inlineStr">
+      <c r="V13" s="4" t="n"/>
+      <c r="W13" s="4" t="n"/>
+      <c r="X13" s="3" t="inlineStr">
         <is>
           <t>SRC-01</t>
         </is>
       </c>
-      <c r="W13" s="3" t="inlineStr">
+      <c r="Y13" s="3" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="X13" s="3" t="n">
+      <c r="Z13" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="Y13" s="3" t="inlineStr">
+      <c r="AA13" s="3" t="inlineStr">
         <is>
           <t>G1A-5</t>
         </is>
       </c>
-      <c r="Z13" s="3" t="n">
+      <c r="AB13" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AA13" s="3" t="n">
+      <c r="AC13" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AB13" s="3" t="n"/>
-      <c r="AC13" s="3" t="n"/>
       <c r="AD13" s="3" t="n"/>
       <c r="AE13" s="3" t="n"/>
       <c r="AF13" s="3" t="n"/>
       <c r="AG13" s="3" t="n"/>
-      <c r="AH13" s="3" t="n">
+      <c r="AH13" s="3" t="n"/>
+      <c r="AI13" s="3" t="n"/>
+      <c r="AJ13" s="3" t="n">
         <v>150</v>
       </c>
-      <c r="AI13" s="3" t="n"/>
-      <c r="AJ13" s="3" t="n"/>
-      <c r="AK13" s="3" t="inlineStr">
+      <c r="AK13" s="3" t="n"/>
+      <c r="AL13" s="3" t="n"/>
+      <c r="AM13" s="3" t="inlineStr">
         <is>
           <t>Upstream source pressure</t>
         </is>
@@ -1654,8 +1712,8 @@
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n"/>
       <c r="K14" s="3" t="n"/>
-      <c r="L14" s="4" t="n"/>
-      <c r="M14" s="4" t="n"/>
+      <c r="L14" s="3" t="n"/>
+      <c r="M14" s="3" t="n"/>
       <c r="N14" s="4" t="n"/>
       <c r="O14" s="4" t="n"/>
       <c r="P14" s="4" t="n"/>
@@ -1664,32 +1722,32 @@
       <c r="S14" s="4" t="n"/>
       <c r="T14" s="4" t="n"/>
       <c r="U14" s="4" t="n"/>
-      <c r="V14" s="3" t="inlineStr">
+      <c r="V14" s="4" t="n"/>
+      <c r="W14" s="4" t="n"/>
+      <c r="X14" s="3" t="inlineStr">
         <is>
           <t>P-301</t>
         </is>
       </c>
-      <c r="W14" s="3" t="inlineStr">
+      <c r="Y14" s="3" t="inlineStr">
         <is>
           <t>Straight Pipeline</t>
         </is>
       </c>
-      <c r="X14" s="3" t="n">
+      <c r="Z14" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="Y14" s="3" t="inlineStr">
+      <c r="AA14" s="3" t="inlineStr">
         <is>
           <t>G1A-5</t>
         </is>
       </c>
-      <c r="Z14" s="3" t="n">
+      <c r="AB14" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="AA14" s="3" t="n">
+      <c r="AC14" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AB14" s="3" t="n"/>
-      <c r="AC14" s="3" t="n"/>
       <c r="AD14" s="3" t="n"/>
       <c r="AE14" s="3" t="n"/>
       <c r="AF14" s="3" t="n"/>
@@ -1697,7 +1755,9 @@
       <c r="AH14" s="3" t="n"/>
       <c r="AI14" s="3" t="n"/>
       <c r="AJ14" s="3" t="n"/>
-      <c r="AK14" s="3" t="inlineStr">
+      <c r="AK14" s="3" t="n"/>
+      <c r="AL14" s="3" t="n"/>
+      <c r="AM14" s="3" t="inlineStr">
         <is>
           <t>Run to valve</t>
         </is>
@@ -1729,8 +1789,8 @@
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
       <c r="K15" s="3" t="n"/>
-      <c r="L15" s="4" t="n"/>
-      <c r="M15" s="4" t="n"/>
+      <c r="L15" s="3" t="n"/>
+      <c r="M15" s="3" t="n"/>
       <c r="N15" s="4" t="n"/>
       <c r="O15" s="4" t="n"/>
       <c r="P15" s="4" t="n"/>
@@ -1739,44 +1799,46 @@
       <c r="S15" s="4" t="n"/>
       <c r="T15" s="4" t="n"/>
       <c r="U15" s="4" t="n"/>
-      <c r="V15" s="3" t="inlineStr">
+      <c r="V15" s="4" t="n"/>
+      <c r="W15" s="4" t="n"/>
+      <c r="X15" s="3" t="inlineStr">
         <is>
           <t>FCV-301</t>
         </is>
       </c>
-      <c r="W15" s="3" t="inlineStr">
+      <c r="Y15" s="3" t="inlineStr">
         <is>
           <t>Control Valve</t>
         </is>
       </c>
-      <c r="X15" s="3" t="n">
+      <c r="Z15" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="Y15" s="3" t="inlineStr">
+      <c r="AA15" s="3" t="inlineStr">
         <is>
           <t>G1A-5</t>
         </is>
       </c>
-      <c r="Z15" s="3" t="n">
+      <c r="AB15" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AA15" s="3" t="n">
+      <c r="AC15" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AB15" s="3" t="n"/>
-      <c r="AC15" s="3" t="n"/>
       <c r="AD15" s="3" t="n"/>
       <c r="AE15" s="3" t="n"/>
       <c r="AF15" s="3" t="n"/>
       <c r="AG15" s="3" t="n"/>
       <c r="AH15" s="3" t="n"/>
-      <c r="AI15" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
+      <c r="AI15" s="3" t="n"/>
       <c r="AJ15" s="3" t="n"/>
       <c r="AK15" s="3" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="AL15" s="3" t="n"/>
+      <c r="AM15" s="3" t="inlineStr">
         <is>
           <t>Flow control — ΔP floats to Destination P</t>
         </is>
@@ -1808,8 +1870,8 @@
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n"/>
       <c r="K16" s="3" t="n"/>
-      <c r="L16" s="4" t="n"/>
-      <c r="M16" s="4" t="n"/>
+      <c r="L16" s="3" t="n"/>
+      <c r="M16" s="3" t="n"/>
       <c r="N16" s="4" t="n"/>
       <c r="O16" s="4" t="n"/>
       <c r="P16" s="4" t="n"/>
@@ -1818,42 +1880,44 @@
       <c r="S16" s="4" t="n"/>
       <c r="T16" s="4" t="n"/>
       <c r="U16" s="4" t="n"/>
-      <c r="V16" s="3" t="inlineStr">
+      <c r="V16" s="4" t="n"/>
+      <c r="W16" s="4" t="n"/>
+      <c r="X16" s="3" t="inlineStr">
         <is>
           <t>DST-01</t>
         </is>
       </c>
-      <c r="W16" s="3" t="inlineStr">
+      <c r="Y16" s="3" t="inlineStr">
         <is>
           <t>Destination</t>
         </is>
       </c>
-      <c r="X16" s="3" t="n">
+      <c r="Z16" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="Y16" s="3" t="inlineStr">
+      <c r="AA16" s="3" t="inlineStr">
         <is>
           <t>G1A-5</t>
         </is>
       </c>
-      <c r="Z16" s="3" t="n">
+      <c r="AB16" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AA16" s="3" t="n">
+      <c r="AC16" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AB16" s="3" t="n"/>
-      <c r="AC16" s="3" t="n"/>
       <c r="AD16" s="3" t="n"/>
       <c r="AE16" s="3" t="n"/>
       <c r="AF16" s="3" t="n"/>
       <c r="AG16" s="3" t="n"/>
-      <c r="AH16" s="3" t="n">
+      <c r="AH16" s="3" t="n"/>
+      <c r="AI16" s="3" t="n"/>
+      <c r="AJ16" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="AI16" s="3" t="n"/>
-      <c r="AJ16" s="3" t="n"/>
-      <c r="AK16" s="3" t="inlineStr">
+      <c r="AK16" s="3" t="n"/>
+      <c r="AL16" s="3" t="n"/>
+      <c r="AM16" s="3" t="inlineStr">
         <is>
           <t>Downstream destination pressure</t>
         </is>
@@ -1889,8 +1953,8 @@
       <c r="I17" s="3" t="n"/>
       <c r="J17" s="3" t="n"/>
       <c r="K17" s="3" t="n"/>
-      <c r="L17" s="4" t="n"/>
-      <c r="M17" s="4" t="n"/>
+      <c r="L17" s="3" t="n"/>
+      <c r="M17" s="3" t="n"/>
       <c r="N17" s="4" t="n"/>
       <c r="O17" s="4" t="n"/>
       <c r="P17" s="4" t="n"/>
@@ -1899,42 +1963,44 @@
       <c r="S17" s="4" t="n"/>
       <c r="T17" s="4" t="n"/>
       <c r="U17" s="4" t="n"/>
-      <c r="V17" s="3" t="inlineStr">
+      <c r="V17" s="4" t="n"/>
+      <c r="W17" s="4" t="n"/>
+      <c r="X17" s="3" t="inlineStr">
         <is>
           <t>SRC-02</t>
         </is>
       </c>
-      <c r="W17" s="3" t="inlineStr">
+      <c r="Y17" s="3" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="X17" s="3" t="n">
+      <c r="Z17" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="Y17" s="3" t="inlineStr">
+      <c r="AA17" s="3" t="inlineStr">
         <is>
           <t>G1A-5</t>
         </is>
       </c>
-      <c r="Z17" s="3" t="n">
+      <c r="AB17" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AA17" s="3" t="n">
+      <c r="AC17" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AB17" s="3" t="n"/>
-      <c r="AC17" s="3" t="n"/>
       <c r="AD17" s="3" t="n"/>
       <c r="AE17" s="3" t="n"/>
       <c r="AF17" s="3" t="n"/>
       <c r="AG17" s="3" t="n"/>
-      <c r="AH17" s="3" t="n">
+      <c r="AH17" s="3" t="n"/>
+      <c r="AI17" s="3" t="n"/>
+      <c r="AJ17" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="AI17" s="3" t="n"/>
-      <c r="AJ17" s="3" t="n"/>
-      <c r="AK17" s="3" t="inlineStr">
+      <c r="AK17" s="3" t="n"/>
+      <c r="AL17" s="3" t="n"/>
+      <c r="AM17" s="3" t="inlineStr">
         <is>
           <t>Header source</t>
         </is>
@@ -1963,13 +2029,13 @@
         <v>2</v>
       </c>
       <c r="H18" s="3" t="n"/>
-      <c r="I18" s="3" t="n">
+      <c r="I18" s="3" t="n"/>
+      <c r="J18" s="3" t="n"/>
+      <c r="K18" s="3" t="n">
         <v>-0.5</v>
       </c>
-      <c r="J18" s="3" t="n"/>
-      <c r="K18" s="3" t="n"/>
-      <c r="L18" s="4" t="n"/>
-      <c r="M18" s="4" t="n"/>
+      <c r="L18" s="3" t="n"/>
+      <c r="M18" s="3" t="n"/>
       <c r="N18" s="4" t="n"/>
       <c r="O18" s="4" t="n"/>
       <c r="P18" s="4" t="n"/>
@@ -1978,32 +2044,32 @@
       <c r="S18" s="4" t="n"/>
       <c r="T18" s="4" t="n"/>
       <c r="U18" s="4" t="n"/>
-      <c r="V18" s="3" t="inlineStr">
+      <c r="V18" s="4" t="n"/>
+      <c r="W18" s="4" t="n"/>
+      <c r="X18" s="3" t="inlineStr">
         <is>
           <t>TEE-40</t>
         </is>
       </c>
-      <c r="W18" s="3" t="inlineStr">
+      <c r="Y18" s="3" t="inlineStr">
         <is>
           <t>Tee Split Branch Flow 1</t>
         </is>
       </c>
-      <c r="X18" s="3" t="n">
+      <c r="Z18" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="Y18" s="3" t="inlineStr">
+      <c r="AA18" s="3" t="inlineStr">
         <is>
           <t>G1A-5</t>
         </is>
       </c>
-      <c r="Z18" s="3" t="n">
+      <c r="AB18" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AA18" s="3" t="n">
+      <c r="AC18" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AB18" s="3" t="n"/>
-      <c r="AC18" s="3" t="n"/>
       <c r="AD18" s="3" t="n"/>
       <c r="AE18" s="3" t="n"/>
       <c r="AF18" s="3" t="n"/>
@@ -2011,7 +2077,9 @@
       <c r="AH18" s="3" t="n"/>
       <c r="AI18" s="3" t="n"/>
       <c r="AJ18" s="3" t="n"/>
-      <c r="AK18" s="3" t="inlineStr">
+      <c r="AK18" s="3" t="n"/>
+      <c r="AL18" s="3" t="n"/>
+      <c r="AM18" s="3" t="inlineStr">
         <is>
           <t>50% splits to parallel branch</t>
         </is>
@@ -2043,8 +2111,8 @@
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
       <c r="K19" s="3" t="n"/>
-      <c r="L19" s="4" t="n"/>
-      <c r="M19" s="4" t="n"/>
+      <c r="L19" s="3" t="n"/>
+      <c r="M19" s="3" t="n"/>
       <c r="N19" s="4" t="n"/>
       <c r="O19" s="4" t="n"/>
       <c r="P19" s="4" t="n"/>
@@ -2053,46 +2121,48 @@
       <c r="S19" s="4" t="n"/>
       <c r="T19" s="4" t="n"/>
       <c r="U19" s="4" t="n"/>
-      <c r="V19" s="3" t="inlineStr">
+      <c r="V19" s="4" t="n"/>
+      <c r="W19" s="4" t="n"/>
+      <c r="X19" s="3" t="inlineStr">
         <is>
           <t>FCV-40A</t>
         </is>
       </c>
-      <c r="W19" s="3" t="inlineStr">
+      <c r="Y19" s="3" t="inlineStr">
         <is>
           <t>Control Valve</t>
         </is>
       </c>
-      <c r="X19" s="3" t="n">
+      <c r="Z19" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="Y19" s="3" t="inlineStr">
+      <c r="AA19" s="3" t="inlineStr">
         <is>
           <t>G1A-5</t>
         </is>
       </c>
-      <c r="Z19" s="3" t="n">
+      <c r="AB19" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AA19" s="3" t="n">
+      <c r="AC19" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AB19" s="3" t="n"/>
-      <c r="AC19" s="3" t="n"/>
-      <c r="AD19" s="3" t="n">
+      <c r="AD19" s="3" t="n"/>
+      <c r="AE19" s="3" t="n"/>
+      <c r="AF19" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="AE19" s="3" t="n"/>
-      <c r="AF19" s="3" t="n"/>
       <c r="AG19" s="3" t="n"/>
       <c r="AH19" s="3" t="n"/>
-      <c r="AI19" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
+      <c r="AI19" s="3" t="n"/>
       <c r="AJ19" s="3" t="n"/>
       <c r="AK19" s="3" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="AL19" s="3" t="n"/>
+      <c r="AM19" s="3" t="inlineStr">
         <is>
           <t>Main-leg valve (50% flow)</t>
         </is>
@@ -2126,8 +2196,8 @@
       <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="n"/>
       <c r="K20" s="3" t="n"/>
-      <c r="L20" s="4" t="n"/>
-      <c r="M20" s="4" t="n"/>
+      <c r="L20" s="3" t="n"/>
+      <c r="M20" s="3" t="n"/>
       <c r="N20" s="4" t="n"/>
       <c r="O20" s="4" t="n"/>
       <c r="P20" s="4" t="n"/>
@@ -2136,65 +2206,67 @@
       <c r="S20" s="4" t="n"/>
       <c r="T20" s="4" t="n"/>
       <c r="U20" s="4" t="n"/>
-      <c r="V20" s="3" t="inlineStr">
+      <c r="V20" s="4" t="n"/>
+      <c r="W20" s="4" t="n"/>
+      <c r="X20" s="3" t="inlineStr">
         <is>
           <t>FCV-40B</t>
         </is>
       </c>
-      <c r="W20" s="3" t="inlineStr">
+      <c r="Y20" s="3" t="inlineStr">
         <is>
           <t>Control Valve</t>
         </is>
       </c>
-      <c r="X20" s="3" t="n">
+      <c r="Z20" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="Y20" s="3" t="inlineStr">
+      <c r="AA20" s="3" t="inlineStr">
         <is>
           <t>G1A-5</t>
         </is>
       </c>
-      <c r="Z20" s="3" t="n">
+      <c r="AB20" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AA20" s="3" t="n">
+      <c r="AC20" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AB20" s="3" t="n"/>
-      <c r="AC20" s="3" t="n"/>
-      <c r="AD20" s="3" t="n">
+      <c r="AD20" s="3" t="n"/>
+      <c r="AE20" s="3" t="n"/>
+      <c r="AF20" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="AE20" s="3" t="n"/>
-      <c r="AF20" s="3" t="n"/>
       <c r="AG20" s="3" t="n"/>
       <c r="AH20" s="3" t="n"/>
-      <c r="AI20" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
+      <c r="AI20" s="3" t="n"/>
       <c r="AJ20" s="3" t="n"/>
       <c r="AK20" s="3" t="inlineStr">
         <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="AL20" s="3" t="n"/>
+      <c r="AM20" s="3" t="inlineStr">
+        <is>
           <t>Parallel-leg valve (other 50% flow)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AK2"/>
+  <autoFilter ref="A2:AM2"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:AK1"/>
+    <mergeCell ref="A1:AM1"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="F3:F2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Main,Branch"</formula1>
     </dataValidation>
-    <dataValidation sqref="AI3:AI2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Control Valve Type" error="F=flow, P=pressure, T=temperature, L=level control" type="list">
+    <dataValidation sqref="AK3:AK2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Control Valve Type" error="F=flow, P=pressure, T=temperature, L=level control" type="list">
       <formula1>"F,P,T,L"</formula1>
     </dataValidation>
-    <dataValidation sqref="W3:W2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Fitting" error="Choose a fitting from the list" type="list">
-      <formula1>_FittingList!$A$1:$A$58</formula1>
+    <dataValidation sqref="Y3:Y2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Fitting" error="Choose a fitting from the list" type="list">
+      <formula1>_FittingList!$A$1:$A$66</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2207,7 +2279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A58"/>
+  <dimension ref="A1:A66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2528,89 +2600,145 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Tee Join Line Flow</t>
+          <t>Tee Join Branch Flow 3</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Tee Split Branch Flow 1</t>
+          <t>Tee Join Branch Flow 4</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Tee Split Branch Flow 2</t>
+          <t>Tee Join Branch Flow 5</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Tee Split Line Flow</t>
+          <t>Tee Join Branch Flow 6</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Fix Pressure</t>
+          <t>Tee Join Line Flow</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Fix K</t>
+          <t>Tee Split Branch Flow 1</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Nozzle</t>
+          <t>Tee Split Branch Flow 2</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Orifice</t>
+          <t>Tee Split Branch Flow 3</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Straight Pipeline</t>
+          <t>Tee Split Branch Flow 4</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Venturi</t>
+          <t>Tee Split Branch Flow 5</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Tee Split Branch Flow 6</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Control Valve</t>
+          <t>Tee Split Line Flow</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
+        <is>
+          <t>Fix Pressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Fix K</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Nozzle</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Orifice</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Straight Pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Venturi</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Control Valve</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
         <is>
           <t>Destination</t>
         </is>
@@ -2627,403 +2755,1582 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A64"/>
+  <dimension ref="A1:I69"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>STREAM COMPOSITION  —  use when NOT referencing an HMB stream.  One COLUMN per phase of each inlet stream; Seq says where it enters the line.  Streams entering at different Seq (or in extra columns) are MIXED.  Component names = HMB 'COMPONENTS' sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Circuit (optional)</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="n"/>
+      <c r="E2" s="7" t="n"/>
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="7" t="n"/>
+      <c r="H2" s="7" t="n"/>
+      <c r="I2" s="7" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Line No</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>H-285</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>H-285</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="n"/>
+      <c r="E3" s="7" t="n"/>
+      <c r="F3" s="7" t="n"/>
+      <c r="G3" s="7" t="n"/>
+      <c r="H3" s="7" t="n"/>
+      <c r="I3" s="7" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Seq</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="7" t="n"/>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="7" t="n"/>
+      <c r="I4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Comp ID (optional)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="7" t="n"/>
+      <c r="E5" s="7" t="n"/>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="n"/>
+      <c r="H5" s="7" t="n"/>
+      <c r="I5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Vapor</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Vapor</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="7" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Basis</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Mass</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Mole</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Phase Flow (lb/hr, mass)</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>amount ↓</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>amount ↓</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>amount ↓</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>amount ↓</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>amount ↓</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>amount ↓</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>amount ↓</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>amount ↓</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>H2</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>METHANE</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>ETHANE</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="7" t="n"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>PROPANE</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>NITROGEN</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="7" t="n"/>
+      <c r="I14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>H2O</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
+      <c r="I15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>H2S</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D17" s="7" t="n"/>
+      <c r="E17" s="7" t="n"/>
+      <c r="F17" s="7" t="n"/>
+      <c r="G17" s="7" t="n"/>
+      <c r="H17" s="7" t="n"/>
+      <c r="I17" s="7" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="n"/>
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="7" t="n"/>
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="7" t="n"/>
+      <c r="I18" s="7" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="n"/>
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="7" t="n"/>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="n"/>
+      <c r="H19" s="7" t="n"/>
+      <c r="I19" s="7" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="n"/>
+      <c r="B20" s="7" t="n"/>
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="7" t="n"/>
+      <c r="E20" s="7" t="n"/>
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="7" t="n"/>
+      <c r="H20" s="7" t="n"/>
+      <c r="I20" s="7" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="n"/>
+      <c r="B21" s="7" t="n"/>
+      <c r="C21" s="7" t="n"/>
+      <c r="D21" s="7" t="n"/>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="7" t="n"/>
+      <c r="H21" s="7" t="n"/>
+      <c r="I21" s="7" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="n"/>
+      <c r="B22" s="7" t="n"/>
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="7" t="n"/>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="7" t="n"/>
+      <c r="G22" s="7" t="n"/>
+      <c r="H22" s="7" t="n"/>
+      <c r="I22" s="7" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="n"/>
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="7" t="n"/>
+      <c r="E23" s="7" t="n"/>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="7" t="n"/>
+      <c r="H23" s="7" t="n"/>
+      <c r="I23" s="7" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="n"/>
+      <c r="B24" s="7" t="n"/>
+      <c r="C24" s="7" t="n"/>
+      <c r="D24" s="7" t="n"/>
+      <c r="E24" s="7" t="n"/>
+      <c r="F24" s="7" t="n"/>
+      <c r="G24" s="7" t="n"/>
+      <c r="H24" s="7" t="n"/>
+      <c r="I24" s="7" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="n"/>
+      <c r="B25" s="7" t="n"/>
+      <c r="C25" s="7" t="n"/>
+      <c r="D25" s="7" t="n"/>
+      <c r="E25" s="7" t="n"/>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="n"/>
+      <c r="H25" s="7" t="n"/>
+      <c r="I25" s="7" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="n"/>
+      <c r="B26" s="7" t="n"/>
+      <c r="C26" s="7" t="n"/>
+      <c r="D26" s="7" t="n"/>
+      <c r="E26" s="7" t="n"/>
+      <c r="F26" s="7" t="n"/>
+      <c r="G26" s="7" t="n"/>
+      <c r="H26" s="7" t="n"/>
+      <c r="I26" s="7" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="n"/>
+      <c r="B27" s="7" t="n"/>
+      <c r="C27" s="7" t="n"/>
+      <c r="D27" s="7" t="n"/>
+      <c r="E27" s="7" t="n"/>
+      <c r="F27" s="7" t="n"/>
+      <c r="G27" s="7" t="n"/>
+      <c r="H27" s="7" t="n"/>
+      <c r="I27" s="7" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="n"/>
+      <c r="B28" s="7" t="n"/>
+      <c r="C28" s="7" t="n"/>
+      <c r="D28" s="7" t="n"/>
+      <c r="E28" s="7" t="n"/>
+      <c r="F28" s="7" t="n"/>
+      <c r="G28" s="7" t="n"/>
+      <c r="H28" s="7" t="n"/>
+      <c r="I28" s="7" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="n"/>
+      <c r="B29" s="7" t="n"/>
+      <c r="C29" s="7" t="n"/>
+      <c r="D29" s="7" t="n"/>
+      <c r="E29" s="7" t="n"/>
+      <c r="F29" s="7" t="n"/>
+      <c r="G29" s="7" t="n"/>
+      <c r="H29" s="7" t="n"/>
+      <c r="I29" s="7" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="n"/>
+      <c r="B30" s="7" t="n"/>
+      <c r="C30" s="7" t="n"/>
+      <c r="D30" s="7" t="n"/>
+      <c r="E30" s="7" t="n"/>
+      <c r="F30" s="7" t="n"/>
+      <c r="G30" s="7" t="n"/>
+      <c r="H30" s="7" t="n"/>
+      <c r="I30" s="7" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="n"/>
+      <c r="B31" s="7" t="n"/>
+      <c r="C31" s="7" t="n"/>
+      <c r="D31" s="7" t="n"/>
+      <c r="E31" s="7" t="n"/>
+      <c r="F31" s="7" t="n"/>
+      <c r="G31" s="7" t="n"/>
+      <c r="H31" s="7" t="n"/>
+      <c r="I31" s="7" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="n"/>
+      <c r="B32" s="7" t="n"/>
+      <c r="C32" s="7" t="n"/>
+      <c r="D32" s="7" t="n"/>
+      <c r="E32" s="7" t="n"/>
+      <c r="F32" s="7" t="n"/>
+      <c r="G32" s="7" t="n"/>
+      <c r="H32" s="7" t="n"/>
+      <c r="I32" s="7" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="n"/>
+      <c r="B33" s="7" t="n"/>
+      <c r="C33" s="7" t="n"/>
+      <c r="D33" s="7" t="n"/>
+      <c r="E33" s="7" t="n"/>
+      <c r="F33" s="7" t="n"/>
+      <c r="G33" s="7" t="n"/>
+      <c r="H33" s="7" t="n"/>
+      <c r="I33" s="7" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="n"/>
+      <c r="B34" s="7" t="n"/>
+      <c r="C34" s="7" t="n"/>
+      <c r="D34" s="7" t="n"/>
+      <c r="E34" s="7" t="n"/>
+      <c r="F34" s="7" t="n"/>
+      <c r="G34" s="7" t="n"/>
+      <c r="H34" s="7" t="n"/>
+      <c r="I34" s="7" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="n"/>
+      <c r="B35" s="7" t="n"/>
+      <c r="C35" s="7" t="n"/>
+      <c r="D35" s="7" t="n"/>
+      <c r="E35" s="7" t="n"/>
+      <c r="F35" s="7" t="n"/>
+      <c r="G35" s="7" t="n"/>
+      <c r="H35" s="7" t="n"/>
+      <c r="I35" s="7" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="n"/>
+      <c r="B36" s="7" t="n"/>
+      <c r="C36" s="7" t="n"/>
+      <c r="D36" s="7" t="n"/>
+      <c r="E36" s="7" t="n"/>
+      <c r="F36" s="7" t="n"/>
+      <c r="G36" s="7" t="n"/>
+      <c r="H36" s="7" t="n"/>
+      <c r="I36" s="7" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="n"/>
+      <c r="B37" s="7" t="n"/>
+      <c r="C37" s="7" t="n"/>
+      <c r="D37" s="7" t="n"/>
+      <c r="E37" s="7" t="n"/>
+      <c r="F37" s="7" t="n"/>
+      <c r="G37" s="7" t="n"/>
+      <c r="H37" s="7" t="n"/>
+      <c r="I37" s="7" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="n"/>
+      <c r="B38" s="7" t="n"/>
+      <c r="C38" s="7" t="n"/>
+      <c r="D38" s="7" t="n"/>
+      <c r="E38" s="7" t="n"/>
+      <c r="F38" s="7" t="n"/>
+      <c r="G38" s="7" t="n"/>
+      <c r="H38" s="7" t="n"/>
+      <c r="I38" s="7" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="n"/>
+      <c r="B39" s="7" t="n"/>
+      <c r="C39" s="7" t="n"/>
+      <c r="D39" s="7" t="n"/>
+      <c r="E39" s="7" t="n"/>
+      <c r="F39" s="7" t="n"/>
+      <c r="G39" s="7" t="n"/>
+      <c r="H39" s="7" t="n"/>
+      <c r="I39" s="7" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="n"/>
+      <c r="B40" s="7" t="n"/>
+      <c r="C40" s="7" t="n"/>
+      <c r="D40" s="7" t="n"/>
+      <c r="E40" s="7" t="n"/>
+      <c r="F40" s="7" t="n"/>
+      <c r="G40" s="7" t="n"/>
+      <c r="H40" s="7" t="n"/>
+      <c r="I40" s="7" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="n"/>
+      <c r="B41" s="7" t="n"/>
+      <c r="C41" s="7" t="n"/>
+      <c r="D41" s="7" t="n"/>
+      <c r="E41" s="7" t="n"/>
+      <c r="F41" s="7" t="n"/>
+      <c r="G41" s="7" t="n"/>
+      <c r="H41" s="7" t="n"/>
+      <c r="I41" s="7" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="n"/>
+      <c r="B42" s="7" t="n"/>
+      <c r="C42" s="7" t="n"/>
+      <c r="D42" s="7" t="n"/>
+      <c r="E42" s="7" t="n"/>
+      <c r="F42" s="7" t="n"/>
+      <c r="G42" s="7" t="n"/>
+      <c r="H42" s="7" t="n"/>
+      <c r="I42" s="7" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="n"/>
+      <c r="B43" s="7" t="n"/>
+      <c r="C43" s="7" t="n"/>
+      <c r="D43" s="7" t="n"/>
+      <c r="E43" s="7" t="n"/>
+      <c r="F43" s="7" t="n"/>
+      <c r="G43" s="7" t="n"/>
+      <c r="H43" s="7" t="n"/>
+      <c r="I43" s="7" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="n"/>
+      <c r="B44" s="7" t="n"/>
+      <c r="C44" s="7" t="n"/>
+      <c r="D44" s="7" t="n"/>
+      <c r="E44" s="7" t="n"/>
+      <c r="F44" s="7" t="n"/>
+      <c r="G44" s="7" t="n"/>
+      <c r="H44" s="7" t="n"/>
+      <c r="I44" s="7" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="n"/>
+      <c r="B45" s="7" t="n"/>
+      <c r="C45" s="7" t="n"/>
+      <c r="D45" s="7" t="n"/>
+      <c r="E45" s="7" t="n"/>
+      <c r="F45" s="7" t="n"/>
+      <c r="G45" s="7" t="n"/>
+      <c r="H45" s="7" t="n"/>
+      <c r="I45" s="7" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="n"/>
+      <c r="B46" s="7" t="n"/>
+      <c r="C46" s="7" t="n"/>
+      <c r="D46" s="7" t="n"/>
+      <c r="E46" s="7" t="n"/>
+      <c r="F46" s="7" t="n"/>
+      <c r="G46" s="7" t="n"/>
+      <c r="H46" s="7" t="n"/>
+      <c r="I46" s="7" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="n"/>
+      <c r="B47" s="7" t="n"/>
+      <c r="C47" s="7" t="n"/>
+      <c r="D47" s="7" t="n"/>
+      <c r="E47" s="7" t="n"/>
+      <c r="F47" s="7" t="n"/>
+      <c r="G47" s="7" t="n"/>
+      <c r="H47" s="7" t="n"/>
+      <c r="I47" s="7" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="n"/>
+      <c r="B48" s="7" t="n"/>
+      <c r="C48" s="7" t="n"/>
+      <c r="D48" s="7" t="n"/>
+      <c r="E48" s="7" t="n"/>
+      <c r="F48" s="7" t="n"/>
+      <c r="G48" s="7" t="n"/>
+      <c r="H48" s="7" t="n"/>
+      <c r="I48" s="7" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="n"/>
+      <c r="B49" s="7" t="n"/>
+      <c r="C49" s="7" t="n"/>
+      <c r="D49" s="7" t="n"/>
+      <c r="E49" s="7" t="n"/>
+      <c r="F49" s="7" t="n"/>
+      <c r="G49" s="7" t="n"/>
+      <c r="H49" s="7" t="n"/>
+      <c r="I49" s="7" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="n"/>
+      <c r="B50" s="7" t="n"/>
+      <c r="C50" s="7" t="n"/>
+      <c r="D50" s="7" t="n"/>
+      <c r="E50" s="7" t="n"/>
+      <c r="F50" s="7" t="n"/>
+      <c r="G50" s="7" t="n"/>
+      <c r="H50" s="7" t="n"/>
+      <c r="I50" s="7" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="n"/>
+      <c r="B51" s="7" t="n"/>
+      <c r="C51" s="7" t="n"/>
+      <c r="D51" s="7" t="n"/>
+      <c r="E51" s="7" t="n"/>
+      <c r="F51" s="7" t="n"/>
+      <c r="G51" s="7" t="n"/>
+      <c r="H51" s="7" t="n"/>
+      <c r="I51" s="7" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="n"/>
+      <c r="B52" s="7" t="n"/>
+      <c r="C52" s="7" t="n"/>
+      <c r="D52" s="7" t="n"/>
+      <c r="E52" s="7" t="n"/>
+      <c r="F52" s="7" t="n"/>
+      <c r="G52" s="7" t="n"/>
+      <c r="H52" s="7" t="n"/>
+      <c r="I52" s="7" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="n"/>
+      <c r="B53" s="7" t="n"/>
+      <c r="C53" s="7" t="n"/>
+      <c r="D53" s="7" t="n"/>
+      <c r="E53" s="7" t="n"/>
+      <c r="F53" s="7" t="n"/>
+      <c r="G53" s="7" t="n"/>
+      <c r="H53" s="7" t="n"/>
+      <c r="I53" s="7" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="n"/>
+      <c r="B54" s="7" t="n"/>
+      <c r="C54" s="7" t="n"/>
+      <c r="D54" s="7" t="n"/>
+      <c r="E54" s="7" t="n"/>
+      <c r="F54" s="7" t="n"/>
+      <c r="G54" s="7" t="n"/>
+      <c r="H54" s="7" t="n"/>
+      <c r="I54" s="7" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="n"/>
+      <c r="B55" s="7" t="n"/>
+      <c r="C55" s="7" t="n"/>
+      <c r="D55" s="7" t="n"/>
+      <c r="E55" s="7" t="n"/>
+      <c r="F55" s="7" t="n"/>
+      <c r="G55" s="7" t="n"/>
+      <c r="H55" s="7" t="n"/>
+      <c r="I55" s="7" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="n"/>
+      <c r="B56" s="7" t="n"/>
+      <c r="C56" s="7" t="n"/>
+      <c r="D56" s="7" t="n"/>
+      <c r="E56" s="7" t="n"/>
+      <c r="F56" s="7" t="n"/>
+      <c r="G56" s="7" t="n"/>
+      <c r="H56" s="7" t="n"/>
+      <c r="I56" s="7" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="10" t="n"/>
+      <c r="B57" s="7" t="n"/>
+      <c r="C57" s="7" t="n"/>
+      <c r="D57" s="7" t="n"/>
+      <c r="E57" s="7" t="n"/>
+      <c r="F57" s="7" t="n"/>
+      <c r="G57" s="7" t="n"/>
+      <c r="H57" s="7" t="n"/>
+      <c r="I57" s="7" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="n"/>
+      <c r="B58" s="7" t="n"/>
+      <c r="C58" s="7" t="n"/>
+      <c r="D58" s="7" t="n"/>
+      <c r="E58" s="7" t="n"/>
+      <c r="F58" s="7" t="n"/>
+      <c r="G58" s="7" t="n"/>
+      <c r="H58" s="7" t="n"/>
+      <c r="I58" s="7" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="10" t="n"/>
+      <c r="B59" s="7" t="n"/>
+      <c r="C59" s="7" t="n"/>
+      <c r="D59" s="7" t="n"/>
+      <c r="E59" s="7" t="n"/>
+      <c r="F59" s="7" t="n"/>
+      <c r="G59" s="7" t="n"/>
+      <c r="H59" s="7" t="n"/>
+      <c r="I59" s="7" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="10" t="n"/>
+      <c r="B60" s="7" t="n"/>
+      <c r="C60" s="7" t="n"/>
+      <c r="D60" s="7" t="n"/>
+      <c r="E60" s="7" t="n"/>
+      <c r="F60" s="7" t="n"/>
+      <c r="G60" s="7" t="n"/>
+      <c r="H60" s="7" t="n"/>
+      <c r="I60" s="7" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="10" t="n"/>
+      <c r="B61" s="7" t="n"/>
+      <c r="C61" s="7" t="n"/>
+      <c r="D61" s="7" t="n"/>
+      <c r="E61" s="7" t="n"/>
+      <c r="F61" s="7" t="n"/>
+      <c r="G61" s="7" t="n"/>
+      <c r="H61" s="7" t="n"/>
+      <c r="I61" s="7" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="10" t="n"/>
+      <c r="B62" s="7" t="n"/>
+      <c r="C62" s="7" t="n"/>
+      <c r="D62" s="7" t="n"/>
+      <c r="E62" s="7" t="n"/>
+      <c r="F62" s="7" t="n"/>
+      <c r="G62" s="7" t="n"/>
+      <c r="H62" s="7" t="n"/>
+      <c r="I62" s="7" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="10" t="n"/>
+      <c r="B63" s="7" t="n"/>
+      <c r="C63" s="7" t="n"/>
+      <c r="D63" s="7" t="n"/>
+      <c r="E63" s="7" t="n"/>
+      <c r="F63" s="7" t="n"/>
+      <c r="G63" s="7" t="n"/>
+      <c r="H63" s="7" t="n"/>
+      <c r="I63" s="7" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="10" t="n"/>
+      <c r="B64" s="7" t="n"/>
+      <c r="C64" s="7" t="n"/>
+      <c r="D64" s="7" t="n"/>
+      <c r="E64" s="7" t="n"/>
+      <c r="F64" s="7" t="n"/>
+      <c r="G64" s="7" t="n"/>
+      <c r="H64" s="7" t="n"/>
+      <c r="I64" s="7" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="10" t="n"/>
+      <c r="B65" s="7" t="n"/>
+      <c r="C65" s="7" t="n"/>
+      <c r="D65" s="7" t="n"/>
+      <c r="E65" s="7" t="n"/>
+      <c r="F65" s="7" t="n"/>
+      <c r="G65" s="7" t="n"/>
+      <c r="H65" s="7" t="n"/>
+      <c r="I65" s="7" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="10" t="n"/>
+      <c r="B66" s="7" t="n"/>
+      <c r="C66" s="7" t="n"/>
+      <c r="D66" s="7" t="n"/>
+      <c r="E66" s="7" t="n"/>
+      <c r="F66" s="7" t="n"/>
+      <c r="G66" s="7" t="n"/>
+      <c r="H66" s="7" t="n"/>
+      <c r="I66" s="7" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="10" t="n"/>
+      <c r="B67" s="7" t="n"/>
+      <c r="C67" s="7" t="n"/>
+      <c r="D67" s="7" t="n"/>
+      <c r="E67" s="7" t="n"/>
+      <c r="F67" s="7" t="n"/>
+      <c r="G67" s="7" t="n"/>
+      <c r="H67" s="7" t="n"/>
+      <c r="I67" s="7" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="10" t="n"/>
+      <c r="B68" s="7" t="n"/>
+      <c r="C68" s="7" t="n"/>
+      <c r="D68" s="7" t="n"/>
+      <c r="E68" s="7" t="n"/>
+      <c r="F68" s="7" t="n"/>
+      <c r="G68" s="7" t="n"/>
+      <c r="H68" s="7" t="n"/>
+      <c r="I68" s="7" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="10" t="n"/>
+      <c r="B69" s="7" t="n"/>
+      <c r="C69" s="7" t="n"/>
+      <c r="D69" s="7" t="n"/>
+      <c r="E69" s="7" t="n"/>
+      <c r="F69" s="7" t="n"/>
+      <c r="G69" s="7" t="n"/>
+      <c r="H69" s="7" t="n"/>
+      <c r="I69" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="B6:AW6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Vapor,Liquid"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B7:AW7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Mass,Mole"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>NO-ISO PIPELINE INPUT — QUICK REFERENCE</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr"/>
+      <c r="A2" s="12" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>CIRCUIT (column A)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  All rows with the same Circuit ID (e.g. C1) are treated as ONE hydraulic series path.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Lines are chained in the ORDER they appear in this sheet.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  The engine produces ONE workbook per circuit.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Stream Lookup, HMB File, Case and Start P need only be filled on the FIRST row of the circuit.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr"/>
+      <c r="A8" s="12" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>HMB FILE &amp; CASE</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  HMB File and Case override the command-line defaults per row (carried forward within a circuit).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  This lets ONE circuit mix multiple streams / cases / HMB workbooks.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  CLI default case is set with  --case "Case 1".</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr"/>
+      <c r="A13" s="12" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>MANUAL STREAM PROPERTIES (yellow cells)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Leave Stream Lookup BLANK to enter properties by hand in the yellow columns.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Fill Temp, Vapor Mass Flow, Vap MW/Visc/Z/Cp-Cv/Density and (optionally) the Liq columns.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  The engine synthesises a frozen flash split from these numbers — no HMB needed.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr"/>
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  OVERRIDE MODE: with Stream Lookup filled (pulling an HMB stream), filling a yellow cell on</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ANY row of that stream makes the typed value win over the HMB property for that field —</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  e.g. type a Vapor Mass Flow to test a different rate without touching the HMB file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  The override persists on every row downstream until changed again or a new stream loads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>FLOW FRACTION FROM MAIN (Tee split / merge)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  On a Tee fitting row, enter a SIGNED fraction of the Main flow:</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    negative  = SPLIT  (that fraction leaves the line)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    positive  = MERGE  (that fraction joins the line)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    negative  = SPLIT   (that fraction of the CURRENT flow leaves the line)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    positive  = MERGE   (running flow becomes that fraction of the ORIGINAL Main flow —</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                         an absolute target, e.g. 0.125 → 0.25 → 0.5 → 1.0 builds a header</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                         up in stages as branches join it)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  The running vapour &amp; liquid mass flows are scaled in Seq order; downstream dP follows.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>MANUAL COMPOSITION  (sheet 'Stream_Composition' — use INSTEAD of an HMB stream)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Each COLUMN is one phase of one inlet stream.  Header rows: Circuit (optional), Line No,</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Seq (where the stream enters), Comp ID (optional, if Seq repeats on a line), Phase</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (Vapor/Liquid), Basis (Mass/Mole — fractions or flows, normalised), Phase Flow (mass).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Component rows use the EXACT names of the HMB 'COMPONENTS' sheet (MW/Tc/Pc/ω are read</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  from the HMB 'COMP_CONSTANTS' sheet, so set HMB File on the row or pass the HMB on the CLI).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Phase Flow blank → the Vapor / Liq Mass Flow cell of that Pipeline_Input row is used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Still type Temp, Vap Z, Vap Visc, Vap Cp/Cv, Liq Density, Liq Visc on that row (yellow);</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MW and the vapour/liquid split come from the composition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MIXING: the first composition on a circuit starts the flow.  Every later column (a later Seq,</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  or another column at the same Seq) is MIXED in: component flows add, the blend is re-flashed</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  and the mixed MW / properties carry downstream.  Provide BOTH a vapour and a liquid column</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  for true K = y/x; with one phase only, Wilson K from the HMB constants is used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="12" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="11" t="inlineStr">
         <is>
           <t>MULTIPLE LINES IN SERIES</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Change Line No to mark a new pipe line.  Keep Circuit the same.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  The outlet pressure of the last component of Line N becomes the inlet pressure of Line N+1.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="12" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
         <is>
           <t>FITTINGS</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Select from the Fitting Name drop-down.  K values applied automatically.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="6" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="12" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="inlineStr">
         <is>
           <t>FIX K  (Fitting = 'Fix K')</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Enter K in the Fixed K column.  Darcy-Weisbach friction and elevation terms still apply.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="12" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="11" t="inlineStr">
         <is>
           <t>FIX PRESSURE  (Fitting = 'Fix Pressure')</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Enter dP (psi) in Fixed dP.  All hydraulics skipped; dP subtracted directly.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="6" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="12" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="11" t="inlineStr">
         <is>
           <t>FLOW ORIFICE  (Instr Type = FO)</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="6" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Set Instr Type = FO.  Enter rated dP in Instr dP (psi).</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="12" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="11" t="inlineStr">
         <is>
           <t>SOURCE / DESTINATION  (boundary fittings)</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Source: enter the upstream pressure in 'Set P (psia)' — it anchors the circuit inlet pressure.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Destination: enter the downstream pressure in 'Set P (psia)' — the target the circuit must reach.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="6" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  If BOTH are filled, a Control Valve placed between them absorbs the pressure difference.</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="6" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  If only one is filled, the pressure is taken from that single value.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="6" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="12" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="11" t="inlineStr">
         <is>
           <t>CONTROL VALVE  (Fitting = 'Control Valve')</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="6" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Set 'Control Valve Type' = F (flow), P (pressure), T (temperature) or L (level).</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="6" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  F (flow): ΔP floats so the running pressure lands on the downstream Destination 'Set P'.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="6" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  P / L: fixed design ΔP — enter it in 'Fixed dP (psi)' (or a resistance in 'Fixed K').</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="6" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  T (temperature): like a fixed ΔP, but floored at 'Exch Max Allow dP (psi)' (exchanger limit).</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="6" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  β ratio = valve Bore (in) ÷ upstream line bore is reported in the Notes column.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="6" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  SERIES valves: place several Control Valve rows in Seq order on the same run.</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="6" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  PARALLEL valves: split flow at a Tee (negative 'Flow Fraction from Main'), put one Control</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="6" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">    Valve on the Main leg and one on a Branch (Run Type = Branch, with its own Start P).</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="6" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="12" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="11" t="inlineStr">
         <is>
           <t>BRANCHES</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="6" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Set Run Type = Branch.  Fill Start P on the first Branch row.</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="6" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Branches are marched independently.  FIV/AIV/regime sheets use the Main run.</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="6" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="12" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="11" t="inlineStr">
+        <is>
+          <t>AUTO-LINKED SPLITS &amp; JOINS (Main ↔ Branch)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  JOIN (Branch → Main): on a Main row, set Fitting = 'Tee Join Branch Flow N'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  The Nth Branch block sharing that row's Line No is auto-matched by ordinal count;</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  its real flashed outlet (flow + composition) is blended into Main at that row — no</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  manual entry needed on the Branch side.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SPLIT (Main → Branch): on a Main row, set Fitting = 'Tee Split Branch Flow N' with a</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  negative 'Flow Fraction from Main'.  The exact flow + composition that leaves Main at</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  that row is captured and auto-fed as the Branch's inlet — the Branch needs no Stream</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lookup or manual properties of its own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Upstream Line No (Branch, optional): which Main Line No this Branch splits from.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Blank → defaults to the most recently seen Main Line No.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Upstream Seq (Branch, optional): the exact Seq of the Main 'Tee Split Branch Flow N' row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Blank → matched by ordinal count, same as the Join side (N = 1, 2, 3 … up to 6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A Branch with no Upstream Line No match falls back to standalone marching (own Stream</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lookup / manual properties / circuit default).</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="12" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="11" t="inlineStr">
         <is>
           <t>UNITS</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="6" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  This workbook is in FPS units (see the UNITS sheet).</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="6" t="inlineStr">
+    <row r="99">
+      <c r="A99" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Change the Unit System cell (or per-quantity overrides) on the UNITS sheet and enter values accordingly —</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="6" t="inlineStr">
+    <row r="100">
+      <c r="A100" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  the engine reads the UNITS sheet and presents all results in the same units.  Bore/NPS is ALWAYS inches.</t>
         </is>
@@ -3034,7 +4341,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C00000"/>
@@ -3051,377 +4358,377 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>UNITS  —  choose FPS or SI; per-quantity overrides optional</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Unit System</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>FPS</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="16" t="inlineStr">
         <is>
           <t>← FPS or SI.  All inputs read &amp; all results written in these units.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Qty code</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>Unit override (optional)</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>Options</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>Pressure (absolute)</t>
         </is>
       </c>
-      <c r="C6" s="13" t="n"/>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="C6" s="19" t="n"/>
+      <c r="D6" s="20" t="inlineStr">
         <is>
           <t>default: psia   |   psia | psig | kPa | kPag | MPa | bara | barg | kg/cm2a | kg/cm2g</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>dP</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>Pressure drop</t>
         </is>
       </c>
-      <c r="C7" s="13" t="n"/>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="C7" s="19" t="n"/>
+      <c r="D7" s="20" t="inlineStr">
         <is>
           <t>default: psi   |   psi | kPa | bar | mbar | kg/cm2</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>Temperature</t>
         </is>
       </c>
-      <c r="C8" s="13" t="n"/>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="C8" s="19" t="n"/>
+      <c r="D8" s="20" t="inlineStr">
         <is>
           <t>default: degF   |   degF | °F | degC | °C | K</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>dT</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>Temperature difference</t>
         </is>
       </c>
-      <c r="C9" s="13" t="n"/>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="C9" s="19" t="n"/>
+      <c r="D9" s="20" t="inlineStr">
         <is>
           <t>default: degF   |   degF | degC | K</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>mflow</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>Mass flow</t>
         </is>
       </c>
-      <c r="C10" s="13" t="n"/>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="C10" s="19" t="n"/>
+      <c r="D10" s="20" t="inlineStr">
         <is>
           <t>default: lb/hr   |   lb/hr | lb/h | kg/hr | kg/h | kg/s | t/h</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>molflow</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>Molar flow</t>
         </is>
       </c>
-      <c r="C11" s="13" t="n"/>
-      <c r="D11" s="14" t="inlineStr">
+      <c r="C11" s="19" t="n"/>
+      <c r="D11" s="20" t="inlineStr">
         <is>
           <t>default: lb-mol/hr   |   lb-mol/hr | kgmol/hr | kmol/h</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>rho</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
         <is>
           <t>Density</t>
         </is>
       </c>
-      <c r="C12" s="13" t="n"/>
-      <c r="D12" s="14" t="inlineStr">
+      <c r="C12" s="19" t="n"/>
+      <c r="D12" s="20" t="inlineStr">
         <is>
           <t>default: lb/ft3   |   lb/ft3 | lb/ft³ | kg/m3 | kg/m³</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>Length / elevation</t>
         </is>
       </c>
-      <c r="C13" s="13" t="n"/>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="C13" s="19" t="n"/>
+      <c r="D13" s="20" t="inlineStr">
         <is>
           <t>default: ft   |   ft | m | mm</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Lin</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>Bore / small length</t>
         </is>
       </c>
-      <c r="C14" s="13" t="n"/>
-      <c r="D14" s="14" t="inlineStr">
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="20" t="inlineStr">
         <is>
           <t>default: in   |   in | mm</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>Surface area</t>
         </is>
       </c>
-      <c r="C15" s="13" t="n"/>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="C15" s="19" t="n"/>
+      <c r="D15" s="20" t="inlineStr">
         <is>
           <t>default: ft2   |   ft2 | ft² | m2 | m²</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>Ain</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="16" t="inlineStr">
         <is>
           <t>Orifice area</t>
         </is>
       </c>
-      <c r="C16" s="13" t="n"/>
-      <c r="D16" s="14" t="inlineStr">
+      <c r="C16" s="19" t="n"/>
+      <c r="D16" s="20" t="inlineStr">
         <is>
           <t>default: in2   |   in2 | in² | cm2 | cm² | mm2 | mm²</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="16" t="inlineStr">
         <is>
           <t>Volume</t>
         </is>
       </c>
-      <c r="C17" s="13" t="n"/>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="C17" s="19" t="n"/>
+      <c r="D17" s="20" t="inlineStr">
         <is>
           <t>default: ft3   |   ft3 | ft³ | m3 | m³ | L</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="16" t="inlineStr">
         <is>
           <t>Heat duty</t>
         </is>
       </c>
-      <c r="C18" s="13" t="n"/>
-      <c r="D18" s="14" t="inlineStr">
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="20" t="inlineStr">
         <is>
           <t>default: BTU/hr   |   BTU/hr | kW | W | MW | MMBTU/hr | kcal/h</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>h</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="16" t="inlineStr">
         <is>
           <t>Specific enthalpy / latent heat</t>
         </is>
       </c>
-      <c r="C19" s="13" t="n"/>
-      <c r="D19" s="14" t="inlineStr">
+      <c r="C19" s="19" t="n"/>
+      <c r="D19" s="20" t="inlineStr">
         <is>
           <t>default: BTU/lb   |   BTU/lb | kJ/kg | kcal/kg</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>v</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="16" t="inlineStr">
         <is>
           <t>Velocity</t>
         </is>
       </c>
-      <c r="C20" s="13" t="n"/>
-      <c r="D20" s="14" t="inlineStr">
+      <c r="C20" s="19" t="n"/>
+      <c r="D20" s="20" t="inlineStr">
         <is>
           <t>default: ft/s   |   ft/s | m/s</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="inlineStr">
+      <c r="A21" s="18" t="inlineStr">
         <is>
           <t>qvol</t>
         </is>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>Volumetric flow</t>
         </is>
       </c>
-      <c r="C21" s="13" t="n"/>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="C21" s="19" t="n"/>
+      <c r="D21" s="20" t="inlineStr">
         <is>
           <t>default: ft3/hr   |   ft3/hr | m3/h | gpm | m3/hr</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="inlineStr">
+      <c r="A22" s="18" t="inlineStr">
         <is>
           <t>visc</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B22" s="16" t="inlineStr">
         <is>
           <t>Viscosity</t>
         </is>
       </c>
-      <c r="C22" s="13" t="n"/>
-      <c r="D22" s="14" t="inlineStr">
+      <c r="C22" s="19" t="n"/>
+      <c r="D22" s="20" t="inlineStr">
         <is>
           <t>default: cP   |   cP</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="inlineStr">
+      <c r="A23" s="18" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B23" s="16" t="inlineStr">
         <is>
           <t>Molecular weight</t>
         </is>
       </c>
-      <c r="C23" s="13" t="n"/>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="C23" s="19" t="n"/>
+      <c r="D23" s="20" t="inlineStr">
         <is>
           <t>default: g/mol   |   g/mol</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="14" t="inlineStr">
+      <c r="A25" s="20" t="inlineStr">
         <is>
           <t>Leave overrides blank to use the system defaults. Overrides apply per quantity (e.g. P = barg while system = SI).</t>
         </is>

</xml_diff>

<commit_message>
Hydraulics: built-in pure-component library (aromatics, paraffins, olefins, oxygenates)
Fallback for composition names absent from the HMB COMP_CONSTANTS sheet; HMB
values always win. Component-name suggestions added to Stream_Composition.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016tUfEsTN4BKrSujrNZ7fBp
</commit_message>
<xml_diff>
--- a/Hydraulics/pipeline_input_noiso.xlsx
+++ b/Hydraulics/pipeline_input_noiso.xlsx
@@ -10,8 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline_Input" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_FittingList" sheetId="2" state="hidden" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stream_Composition" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UNITS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_CompList" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UNITS" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pipeline_Input'!$A$2:$AM$2</definedName>
@@ -3672,7 +3673,10 @@
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="3">
+    <dataValidation sqref="A10:A200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>_CompList!$A$1:$A$57</formula1>
+    </dataValidation>
     <dataValidation sqref="B6:AW6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Vapor,Liquid"</formula1>
     </dataValidation>
@@ -3690,7 +3694,420 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A100"/>
+  <dimension ref="A1:A57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>H2O</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>H2S</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NH3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>H2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NITROGEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>METHANE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ETHANE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PROPANE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>IC4</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>NC4</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>IC5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>NC5</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CYCLOPENTANE</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ISOHEXANE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>HCL</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SO2</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SO3</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CL2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>O2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BENZENE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TOLUENE</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ETHYLBENZENE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>O-XYLENE</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>M-XYLENE</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>P-XYLENE</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>STYRENE</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>CUMENE</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>N-PROPYLBENZENE</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>124TMB</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>135TMB</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>N-BUTYLBENZENE</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NAPHTHALENE</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>1-METHYLNAPHTHALENE</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>BIPHENYL</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>NC6</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>NC7</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>NC8</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>NC9</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>NC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>NC12</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>NC16</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>CYCLOHEXANE</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>METHYLCYCLOPENTANE</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>METHYLCYCLOHEXANE</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ETHYLENE</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>PROPYLENE</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>1-BUTENE</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ISOBUTYLENE</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>BUTADIENE</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ACETYLENE</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>HELIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ARGON</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>METHANOL</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>ETHANOL</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>PHENOL</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -3931,90 +4348,94 @@
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Phase Flow blank → the Vapor / Liq Mass Flow cell of that Pipeline_Input row is used.</t>
+          <t xml:space="preserve">  Names missing from the HMB fall back to a built-in PURE library (benzene, toluene, xylenes,</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Still type Temp, Vap Z, Vap Visc, Vap Cp/Cv, Liq Density, Liq Visc on that row (yellow);</t>
+          <t xml:space="preserve">  styrene, cumene, trimethylbenzenes, butylbenzene, naphthalene, methylnaphthalene, biphenyl,</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MW and the vapour/liquid split come from the composition.</t>
+          <t xml:space="preserve">  NC6-NC16, cyclohexanes, olefins, He/Ar, methanol/ethanol/phenol — see _PURE_LIB_ROWS).</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MIXING: the first composition on a circuit starts the flow.  Every later column (a later Seq,</t>
+          <t xml:space="preserve">  Phase Flow blank → the Vapor / Liq Mass Flow cell of that Pipeline_Input row is used.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  or another column at the same Seq) is MIXED in: component flows add, the blend is re-flashed</t>
+          <t xml:space="preserve">  Still type Temp, Vap Z, Vap Visc, Vap Cp/Cv, Liq Density, Liq Visc on that row (yellow);</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  and the mixed MW / properties carry downstream.  Provide BOTH a vapour and a liquid column</t>
+          <t xml:space="preserve">  MW and the vapour/liquid split come from the composition.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  for true K = y/x; with one phase only, Wilson K from the HMB constants is used.</t>
+          <t xml:space="preserve">  MIXING: the first composition on a circuit starts the flow.  Every later column (a later Seq,</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="12" t="inlineStr"/>
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  or another column at the same Seq) is MIXED in: component flows add, the blend is re-flashed</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="11" t="inlineStr">
-        <is>
-          <t>MULTIPLE LINES IN SERIES</t>
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  and the mixed MW / properties carry downstream.  Provide BOTH a vapour and a liquid column</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">  for true K = y/x; with one phase only, Wilson K from the HMB constants is used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="12" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="inlineStr">
+        <is>
+          <t>MULTIPLE LINES IN SERIES</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Change Line No to mark a new pipe line.  Keep Circuit the same.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  The outlet pressure of the last component of Line N becomes the inlet pressure of Line N+1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="12" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="11" t="inlineStr">
-        <is>
-          <t>FITTINGS</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Select from the Fitting Name drop-down.  K values applied automatically.</t>
+          <t xml:space="preserve">  The outlet pressure of the last component of Line N becomes the inlet pressure of Line N+1.</t>
         </is>
       </c>
     </row>
@@ -4024,14 +4445,14 @@
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
         <is>
-          <t>FIX K  (Fitting = 'Fix K')</t>
+          <t>FITTINGS</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Enter K in the Fixed K column.  Darcy-Weisbach friction and elevation terms still apply.</t>
+          <t xml:space="preserve">  Select from the Fitting Name drop-down.  K values applied automatically.</t>
         </is>
       </c>
     </row>
@@ -4041,14 +4462,14 @@
     <row r="55">
       <c r="A55" s="11" t="inlineStr">
         <is>
-          <t>FIX PRESSURE  (Fitting = 'Fix Pressure')</t>
+          <t>FIX K  (Fitting = 'Fix K')</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Enter dP (psi) in Fixed dP.  All hydraulics skipped; dP subtracted directly.</t>
+          <t xml:space="preserve">  Enter K in the Fixed K column.  Darcy-Weisbach friction and elevation terms still apply.</t>
         </is>
       </c>
     </row>
@@ -4058,14 +4479,14 @@
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
         <is>
-          <t>FLOW ORIFICE  (Instr Type = FO)</t>
+          <t>FIX PRESSURE  (Fitting = 'Fix Pressure')</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Set Instr Type = FO.  Enter rated dP in Instr dP (psi).</t>
+          <t xml:space="preserve">  Enter dP (psi) in Fixed dP.  All hydraulics skipped; dP subtracted directly.</t>
         </is>
       </c>
     </row>
@@ -4075,262 +4496,279 @@
     <row r="61">
       <c r="A61" s="11" t="inlineStr">
         <is>
-          <t>SOURCE / DESTINATION  (boundary fittings)</t>
+          <t>FLOW ORIFICE  (Instr Type = FO)</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Source: enter the upstream pressure in 'Set P (psia)' — it anchors the circuit inlet pressure.</t>
+          <t xml:space="preserve">  Set Instr Type = FO.  Enter rated dP in Instr dP (psi).</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Destination: enter the downstream pressure in 'Set P (psia)' — the target the circuit must reach.</t>
-        </is>
-      </c>
+      <c r="A63" s="12" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  If BOTH are filled, a Control Valve placed between them absorbs the pressure difference.</t>
+      <c r="A64" s="11" t="inlineStr">
+        <is>
+          <t>SOURCE / DESTINATION  (boundary fittings)</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  If only one is filled, the pressure is taken from that single value.</t>
+          <t xml:space="preserve">  Source: enter the upstream pressure in 'Set P (psia)' — it anchors the circuit inlet pressure.</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="12" t="inlineStr"/>
+      <c r="A66" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Destination: enter the downstream pressure in 'Set P (psia)' — the target the circuit must reach.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
-      <c r="A67" s="11" t="inlineStr">
-        <is>
-          <t>CONTROL VALVE  (Fitting = 'Control Valve')</t>
+      <c r="A67" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  If BOTH are filled, a Control Valve placed between them absorbs the pressure difference.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Set 'Control Valve Type' = F (flow), P (pressure), T (temperature) or L (level).</t>
+          <t xml:space="preserve">  If only one is filled, the pressure is taken from that single value.</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  F (flow): ΔP floats so the running pressure lands on the downstream Destination 'Set P'.</t>
-        </is>
-      </c>
+      <c r="A69" s="12" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  P / L: fixed design ΔP — enter it in 'Fixed dP (psi)' (or a resistance in 'Fixed K').</t>
+      <c r="A70" s="11" t="inlineStr">
+        <is>
+          <t>CONTROL VALVE  (Fitting = 'Control Valve')</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  T (temperature): like a fixed ΔP, but floored at 'Exch Max Allow dP (psi)' (exchanger limit).</t>
+          <t xml:space="preserve">  Set 'Control Valve Type' = F (flow), P (pressure), T (temperature) or L (level).</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  β ratio = valve Bore (in) ÷ upstream line bore is reported in the Notes column.</t>
+          <t xml:space="preserve">  F (flow): ΔP floats so the running pressure lands on the downstream Destination 'Set P'.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SERIES valves: place several Control Valve rows in Seq order on the same run.</t>
+          <t xml:space="preserve">  P / L: fixed design ΔP — enter it in 'Fixed dP (psi)' (or a resistance in 'Fixed K').</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  PARALLEL valves: split flow at a Tee (negative 'Flow Fraction from Main'), put one Control</t>
+          <t xml:space="preserve">  T (temperature): like a fixed ΔP, but floored at 'Exch Max Allow dP (psi)' (exchanger limit).</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Valve on the Main leg and one on a Branch (Run Type = Branch, with its own Start P).</t>
+          <t xml:space="preserve">  β ratio = valve Bore (in) ÷ upstream line bore is reported in the Notes column.</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="12" t="inlineStr"/>
+      <c r="A76" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SERIES valves: place several Control Valve rows in Seq order on the same run.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" s="11" t="inlineStr">
-        <is>
-          <t>BRANCHES</t>
+      <c r="A77" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PARALLEL valves: split flow at a Tee (negative 'Flow Fraction from Main'), put one Control</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">    Valve on the Main leg and one on a Branch (Run Type = Branch, with its own Start P).</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="12" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="inlineStr">
+        <is>
+          <t>BRANCHES</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Set Run Type = Branch.  Fill Start P on the first Branch row.</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Branches are marched independently.  FIV/AIV/regime sheets use the Main run.</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="12" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="11" t="inlineStr">
-        <is>
-          <t>AUTO-LINKED SPLITS &amp; JOINS (Main ↔ Branch)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  JOIN (Branch → Main): on a Main row, set Fitting = 'Tee Join Branch Flow N'.</t>
+          <t xml:space="preserve">  Branches are marched independently.  FIV/AIV/regime sheets use the Main run.</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  The Nth Branch block sharing that row's Line No is auto-matched by ordinal count;</t>
-        </is>
-      </c>
+      <c r="A83" s="12" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  its real flashed outlet (flow + composition) is blended into Main at that row — no</t>
+      <c r="A84" s="11" t="inlineStr">
+        <is>
+          <t>AUTO-LINKED SPLITS &amp; JOINS (Main ↔ Branch)</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  manual entry needed on the Branch side.</t>
+          <t xml:space="preserve">  JOIN (Branch → Main): on a Main row, set Fitting = 'Tee Join Branch Flow N'.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SPLIT (Main → Branch): on a Main row, set Fitting = 'Tee Split Branch Flow N' with a</t>
+          <t xml:space="preserve">  The Nth Branch block sharing that row's Line No is auto-matched by ordinal count;</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  negative 'Flow Fraction from Main'.  The exact flow + composition that leaves Main at</t>
+          <t xml:space="preserve">  its real flashed outlet (flow + composition) is blended into Main at that row — no</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  that row is captured and auto-fed as the Branch's inlet — the Branch needs no Stream</t>
+          <t xml:space="preserve">  manual entry needed on the Branch side.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Lookup or manual properties of its own.</t>
+          <t xml:space="preserve">  SPLIT (Main → Branch): on a Main row, set Fitting = 'Tee Split Branch Flow N' with a</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Upstream Line No (Branch, optional): which Main Line No this Branch splits from.</t>
+          <t xml:space="preserve">  negative 'Flow Fraction from Main'.  The exact flow + composition that leaves Main at</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Blank → defaults to the most recently seen Main Line No.</t>
+          <t xml:space="preserve">  that row is captured and auto-fed as the Branch's inlet — the Branch needs no Stream</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Upstream Seq (Branch, optional): the exact Seq of the Main 'Tee Split Branch Flow N' row.</t>
+          <t xml:space="preserve">  Lookup or manual properties of its own.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Blank → matched by ordinal count, same as the Join side (N = 1, 2, 3 … up to 6).</t>
+          <t xml:space="preserve">  Upstream Line No (Branch, optional): which Main Line No this Branch splits from.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  A Branch with no Upstream Line No match falls back to standalone marching (own Stream</t>
+          <t xml:space="preserve">    Blank → defaults to the most recently seen Main Line No.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Lookup / manual properties / circuit default).</t>
+          <t xml:space="preserve">  Upstream Seq (Branch, optional): the exact Seq of the Main 'Tee Split Branch Flow N' row.</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="12" t="inlineStr"/>
+      <c r="A96" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Blank → matched by ordinal count, same as the Join side (N = 1, 2, 3 … up to 6).</t>
+        </is>
+      </c>
     </row>
     <row r="97">
-      <c r="A97" s="11" t="inlineStr">
-        <is>
-          <t>UNITS</t>
+      <c r="A97" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A Branch with no Upstream Line No match falls back to standalone marching (own Stream</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Lookup / manual properties / circuit default).</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="12" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="11" t="inlineStr">
+        <is>
+          <t>UNITS</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">  This workbook is in FPS units (see the UNITS sheet).</t>
         </is>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="12" t="inlineStr">
+    <row r="102">
+      <c r="A102" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Change the Unit System cell (or per-quantity overrides) on the UNITS sheet and enter values accordingly —</t>
         </is>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="12" t="inlineStr">
+    <row r="103">
+      <c r="A103" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  the engine reads the UNITS sheet and presents all results in the same units.  Bore/NPS is ALWAYS inches.</t>
         </is>
@@ -4341,7 +4779,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C00000"/>

</xml_diff>

<commit_message>
Hydraulics: property estimation from Tb/SG/MW and pseudo-component sheet
- Estimate vapor/liquid viscosity, Z, Cp, Cp/Cv, k, sigma, liquid density and
  enthalpy by generalised correlations where no input/HMB value exists; used by
  the hydraulics for composition streams and shown (flagged) in Component_Detail.
- Pseudo_Components input sheet: define a component from MW, NBP, SG; Tc/Pc via
  Exxon-style polynomial, omega via Edmister, optional overrides.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016tUfEsTN4BKrSujrNZ7fBp
</commit_message>
<xml_diff>
--- a/Hydraulics/pipeline_input_noiso.xlsx
+++ b/Hydraulics/pipeline_input_noiso.xlsx
@@ -11,8 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_FittingList" sheetId="2" state="hidden" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stream_Composition" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_CompList" sheetId="4" state="hidden" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UNITS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pseudo_Components" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UNITS" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pipeline_Input'!$A$2:$AM$2</definedName>
@@ -4107,7 +4108,424 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A103"/>
+  <dimension ref="A1:G39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PSEUDO-COMPONENTS — define a component the HMB does not have from MW, NBP and SG.  Tc, Pc (Exxon-style correlation) and ω (Edmister) are estimated; type Tc / Pc / ω only to override.  Use the Name in Stream_Composition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>MW (g/mol)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>NBP (°F)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>SG (60/60°F)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Tc (°F) [opt]</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Pc (psia) [opt]</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>ω [opt]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>HVY_AROM_C11</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>143</v>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>490</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>0.97</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>HVY_AROM_C14</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>184</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>620</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n"/>
+      <c r="B5" s="7" t="n"/>
+      <c r="C5" s="7" t="n"/>
+      <c r="D5" s="7" t="n"/>
+      <c r="E5" s="7" t="n"/>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="n"/>
+      <c r="B6" s="7" t="n"/>
+      <c r="C6" s="7" t="n"/>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n"/>
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n"/>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n"/>
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n"/>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n"/>
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n"/>
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="7" t="n"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n"/>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="n"/>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n"/>
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n"/>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="n"/>
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="7" t="n"/>
+      <c r="E17" s="7" t="n"/>
+      <c r="F17" s="7" t="n"/>
+      <c r="G17" s="7" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="n"/>
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="7" t="n"/>
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="n"/>
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="7" t="n"/>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="n"/>
+      <c r="B20" s="7" t="n"/>
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="7" t="n"/>
+      <c r="E20" s="7" t="n"/>
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="7" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="n"/>
+      <c r="B21" s="7" t="n"/>
+      <c r="C21" s="7" t="n"/>
+      <c r="D21" s="7" t="n"/>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="7" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="n"/>
+      <c r="B22" s="7" t="n"/>
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="7" t="n"/>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="7" t="n"/>
+      <c r="G22" s="7" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="n"/>
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="7" t="n"/>
+      <c r="E23" s="7" t="n"/>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="7" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="n"/>
+      <c r="B24" s="7" t="n"/>
+      <c r="C24" s="7" t="n"/>
+      <c r="D24" s="7" t="n"/>
+      <c r="E24" s="7" t="n"/>
+      <c r="F24" s="7" t="n"/>
+      <c r="G24" s="7" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="n"/>
+      <c r="B25" s="7" t="n"/>
+      <c r="C25" s="7" t="n"/>
+      <c r="D25" s="7" t="n"/>
+      <c r="E25" s="7" t="n"/>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="n"/>
+      <c r="B26" s="7" t="n"/>
+      <c r="C26" s="7" t="n"/>
+      <c r="D26" s="7" t="n"/>
+      <c r="E26" s="7" t="n"/>
+      <c r="F26" s="7" t="n"/>
+      <c r="G26" s="7" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="n"/>
+      <c r="B27" s="7" t="n"/>
+      <c r="C27" s="7" t="n"/>
+      <c r="D27" s="7" t="n"/>
+      <c r="E27" s="7" t="n"/>
+      <c r="F27" s="7" t="n"/>
+      <c r="G27" s="7" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="n"/>
+      <c r="B28" s="7" t="n"/>
+      <c r="C28" s="7" t="n"/>
+      <c r="D28" s="7" t="n"/>
+      <c r="E28" s="7" t="n"/>
+      <c r="F28" s="7" t="n"/>
+      <c r="G28" s="7" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="n"/>
+      <c r="B29" s="7" t="n"/>
+      <c r="C29" s="7" t="n"/>
+      <c r="D29" s="7" t="n"/>
+      <c r="E29" s="7" t="n"/>
+      <c r="F29" s="7" t="n"/>
+      <c r="G29" s="7" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="n"/>
+      <c r="B30" s="7" t="n"/>
+      <c r="C30" s="7" t="n"/>
+      <c r="D30" s="7" t="n"/>
+      <c r="E30" s="7" t="n"/>
+      <c r="F30" s="7" t="n"/>
+      <c r="G30" s="7" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="n"/>
+      <c r="B31" s="7" t="n"/>
+      <c r="C31" s="7" t="n"/>
+      <c r="D31" s="7" t="n"/>
+      <c r="E31" s="7" t="n"/>
+      <c r="F31" s="7" t="n"/>
+      <c r="G31" s="7" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="n"/>
+      <c r="B32" s="7" t="n"/>
+      <c r="C32" s="7" t="n"/>
+      <c r="D32" s="7" t="n"/>
+      <c r="E32" s="7" t="n"/>
+      <c r="F32" s="7" t="n"/>
+      <c r="G32" s="7" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="n"/>
+      <c r="B33" s="7" t="n"/>
+      <c r="C33" s="7" t="n"/>
+      <c r="D33" s="7" t="n"/>
+      <c r="E33" s="7" t="n"/>
+      <c r="F33" s="7" t="n"/>
+      <c r="G33" s="7" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="n"/>
+      <c r="B34" s="7" t="n"/>
+      <c r="C34" s="7" t="n"/>
+      <c r="D34" s="7" t="n"/>
+      <c r="E34" s="7" t="n"/>
+      <c r="F34" s="7" t="n"/>
+      <c r="G34" s="7" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="n"/>
+      <c r="B35" s="7" t="n"/>
+      <c r="C35" s="7" t="n"/>
+      <c r="D35" s="7" t="n"/>
+      <c r="E35" s="7" t="n"/>
+      <c r="F35" s="7" t="n"/>
+      <c r="G35" s="7" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="n"/>
+      <c r="B36" s="7" t="n"/>
+      <c r="C36" s="7" t="n"/>
+      <c r="D36" s="7" t="n"/>
+      <c r="E36" s="7" t="n"/>
+      <c r="F36" s="7" t="n"/>
+      <c r="G36" s="7" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="n"/>
+      <c r="B37" s="7" t="n"/>
+      <c r="C37" s="7" t="n"/>
+      <c r="D37" s="7" t="n"/>
+      <c r="E37" s="7" t="n"/>
+      <c r="F37" s="7" t="n"/>
+      <c r="G37" s="7" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="n"/>
+      <c r="B38" s="7" t="n"/>
+      <c r="C38" s="7" t="n"/>
+      <c r="D38" s="7" t="n"/>
+      <c r="E38" s="7" t="n"/>
+      <c r="F38" s="7" t="n"/>
+      <c r="G38" s="7" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="n"/>
+      <c r="B39" s="7" t="n"/>
+      <c r="C39" s="7" t="n"/>
+      <c r="D39" s="7" t="n"/>
+      <c r="E39" s="7" t="n"/>
+      <c r="F39" s="7" t="n"/>
+      <c r="G39" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -4348,427 +4766,441 @@
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Names missing from the HMB fall back to a built-in PURE library (benzene, toluene, xylenes,</t>
+          <t xml:space="preserve">  PSEUDO-COMPONENTS: define any extra component on the 'Pseudo_Components' sheet from MW, NBP</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  styrene, cumene, trimethylbenzenes, butylbenzene, naphthalene, methylnaphthalene, biphenyl,</t>
+          <t xml:space="preserve">  and SG (Tc/Pc via Exxon-style correlation, ω via Edmister); then use its Name here.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NC6-NC16, cyclohexanes, olefins, He/Ar, methanol/ethanol/phenol — see _PURE_LIB_ROWS).</t>
+          <t xml:space="preserve">  Names missing from the HMB fall back to a built-in PURE library (benzene, toluene, xylenes,</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Phase Flow blank → the Vapor / Liq Mass Flow cell of that Pipeline_Input row is used.</t>
+          <t xml:space="preserve">  styrene, cumene, trimethylbenzenes, butylbenzene, naphthalene, methylnaphthalene, biphenyl,</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Still type Temp, Vap Z, Vap Visc, Vap Cp/Cv, Liq Density, Liq Visc on that row (yellow);</t>
+          <t xml:space="preserve">  NC6-NC16, cyclohexanes, olefins, He/Ar, methanol/ethanol/phenol — see _PURE_LIB_ROWS).</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MW and the vapour/liquid split come from the composition.</t>
+          <t xml:space="preserve">  Phase Flow blank → the Vapor / Liq Mass Flow cell of that Pipeline_Input row is used.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MIXING: the first composition on a circuit starts the flow.  Every later column (a later Seq,</t>
+          <t xml:space="preserve">  Still type Temp, Vap Z, Vap Visc, Vap Cp/Cv, Liq Density, Liq Visc on that row (yellow);</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  or another column at the same Seq) is MIXED in: component flows add, the blend is re-flashed</t>
+          <t xml:space="preserve">  MW and the vapour/liquid split come from the composition.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  and the mixed MW / properties carry downstream.  Provide BOTH a vapour and a liquid column</t>
+          <t xml:space="preserve">  MIXING: the first composition on a circuit starts the flow.  Every later column (a later Seq,</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">  or another column at the same Seq) is MIXED in: component flows add, the blend is re-flashed</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  and the mixed MW / properties carry downstream.  Provide BOTH a vapour and a liquid column</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">  for true K = y/x; with one phase only, Wilson K from the HMB constants is used.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="12" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="11" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="12" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="inlineStr">
         <is>
           <t>MULTIPLE LINES IN SERIES</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="12" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Change Line No to mark a new pipe line.  Keep Circuit the same.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="12" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  The outlet pressure of the last component of Line N becomes the inlet pressure of Line N+1.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="12" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="11" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="12" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="11" t="inlineStr">
         <is>
           <t>FITTINGS</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="12" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Select from the Fitting Name drop-down.  K values applied automatically.</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="12" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="11" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="12" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="11" t="inlineStr">
         <is>
           <t>FIX K  (Fitting = 'Fix K')</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="12" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Enter K in the Fixed K column.  Darcy-Weisbach friction and elevation terms still apply.</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="12" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="11" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="12" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
         <is>
           <t>FIX PRESSURE  (Fitting = 'Fix Pressure')</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="12" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Enter dP (psi) in Fixed dP.  All hydraulics skipped; dP subtracted directly.</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="12" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="11" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="12" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="11" t="inlineStr">
         <is>
           <t>FLOW ORIFICE  (Instr Type = FO)</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="12" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Set Instr Type = FO.  Enter rated dP in Instr dP (psi).</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="12" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="11" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="12" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="inlineStr">
         <is>
           <t>SOURCE / DESTINATION  (boundary fittings)</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Source: enter the upstream pressure in 'Set P (psia)' — it anchors the circuit inlet pressure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Destination: enter the downstream pressure in 'Set P (psia)' — the target the circuit must reach.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  If BOTH are filled, a Control Valve placed between them absorbs the pressure difference.</t>
+          <t xml:space="preserve">  Source: enter the upstream pressure in 'Set P (psia)' — it anchors the circuit inlet pressure.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Destination: enter the downstream pressure in 'Set P (psia)' — the target the circuit must reach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  If BOTH are filled, a Control Valve placed between them absorbs the pressure difference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">  If only one is filled, the pressure is taken from that single value.</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="12" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="11" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="12" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="inlineStr">
         <is>
           <t>CONTROL VALVE  (Fitting = 'Control Valve')</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Set 'Control Valve Type' = F (flow), P (pressure), T (temperature) or L (level).</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  F (flow): ΔP floats so the running pressure lands on the downstream Destination 'Set P'.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  P / L: fixed design ΔP — enter it in 'Fixed dP (psi)' (or a resistance in 'Fixed K').</t>
+          <t xml:space="preserve">  Set 'Control Valve Type' = F (flow), P (pressure), T (temperature) or L (level).</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  T (temperature): like a fixed ΔP, but floored at 'Exch Max Allow dP (psi)' (exchanger limit).</t>
+          <t xml:space="preserve">  F (flow): ΔP floats so the running pressure lands on the downstream Destination 'Set P'.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  β ratio = valve Bore (in) ÷ upstream line bore is reported in the Notes column.</t>
+          <t xml:space="preserve">  P / L: fixed design ΔP — enter it in 'Fixed dP (psi)' (or a resistance in 'Fixed K').</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SERIES valves: place several Control Valve rows in Seq order on the same run.</t>
+          <t xml:space="preserve">  T (temperature): like a fixed ΔP, but floored at 'Exch Max Allow dP (psi)' (exchanger limit).</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  PARALLEL valves: split flow at a Tee (negative 'Flow Fraction from Main'), put one Control</t>
+          <t xml:space="preserve">  β ratio = valve Bore (in) ÷ upstream line bore is reported in the Notes column.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">  SERIES valves: place several Control Valve rows in Seq order on the same run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PARALLEL valves: split flow at a Tee (negative 'Flow Fraction from Main'), put one Control</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">    Valve on the Main leg and one on a Branch (Run Type = Branch, with its own Start P).</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="12" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="11" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="12" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="inlineStr">
         <is>
           <t>BRANCHES</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="12" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Set Run Type = Branch.  Fill Start P on the first Branch row.</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="12" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  Branches are marched independently.  FIV/AIV/regime sheets use the Main run.</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="12" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="11" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="12" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="11" t="inlineStr">
         <is>
           <t>AUTO-LINKED SPLITS &amp; JOINS (Main ↔ Branch)</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  JOIN (Branch → Main): on a Main row, set Fitting = 'Tee Join Branch Flow N'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  The Nth Branch block sharing that row's Line No is auto-matched by ordinal count;</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  its real flashed outlet (flow + composition) is blended into Main at that row — no</t>
+          <t xml:space="preserve">  JOIN (Branch → Main): on a Main row, set Fitting = 'Tee Join Branch Flow N'.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  manual entry needed on the Branch side.</t>
+          <t xml:space="preserve">  The Nth Branch block sharing that row's Line No is auto-matched by ordinal count;</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SPLIT (Main → Branch): on a Main row, set Fitting = 'Tee Split Branch Flow N' with a</t>
+          <t xml:space="preserve">  its real flashed outlet (flow + composition) is blended into Main at that row — no</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  negative 'Flow Fraction from Main'.  The exact flow + composition that leaves Main at</t>
+          <t xml:space="preserve">  manual entry needed on the Branch side.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  that row is captured and auto-fed as the Branch's inlet — the Branch needs no Stream</t>
+          <t xml:space="preserve">  SPLIT (Main → Branch): on a Main row, set Fitting = 'Tee Split Branch Flow N' with a</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Lookup or manual properties of its own.</t>
+          <t xml:space="preserve">  negative 'Flow Fraction from Main'.  The exact flow + composition that leaves Main at</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Upstream Line No (Branch, optional): which Main Line No this Branch splits from.</t>
+          <t xml:space="preserve">  that row is captured and auto-fed as the Branch's inlet — the Branch needs no Stream</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Blank → defaults to the most recently seen Main Line No.</t>
+          <t xml:space="preserve">  Lookup or manual properties of its own.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Upstream Seq (Branch, optional): the exact Seq of the Main 'Tee Split Branch Flow N' row.</t>
+          <t xml:space="preserve">  Upstream Line No (Branch, optional): which Main Line No this Branch splits from.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Blank → matched by ordinal count, same as the Join side (N = 1, 2, 3 … up to 6).</t>
+          <t xml:space="preserve">    Blank → defaults to the most recently seen Main Line No.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  A Branch with no Upstream Line No match falls back to standalone marching (own Stream</t>
+          <t xml:space="preserve">  Upstream Seq (Branch, optional): the exact Seq of the Main 'Tee Split Branch Flow N' row.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">    Blank → matched by ordinal count, same as the Join side (N = 1, 2, 3 … up to 6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A Branch with no Upstream Line No match falls back to standalone marching (own Stream</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Lookup / manual properties / circuit default).</t>
         </is>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="12" t="inlineStr"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="11" t="inlineStr">
+    <row r="101">
+      <c r="A101" s="12" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="11" t="inlineStr">
         <is>
           <t>UNITS</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  This workbook is in FPS units (see the UNITS sheet).</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Change the Unit System cell (or per-quantity overrides) on the UNITS sheet and enter values accordingly —</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  This workbook is in FPS units (see the UNITS sheet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Change the Unit System cell (or per-quantity overrides) on the UNITS sheet and enter values accordingly —</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  the engine reads the UNITS sheet and presents all results in the same units.  Bore/NPS is ALWAYS inches.</t>
         </is>
@@ -4779,7 +5211,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C00000"/>

</xml_diff>